<commit_message>
Separate SAP E01 from AS400 and rewrite workbook copy
SAP E01 was being treated as the umbrella scope of the whole list: it
appeared in the title banner and doubled as AS400's functional area,
which implied AS400 was a SAP application. They are unrelated systems.

- SAP E01 is now its own row (1), area "SAP / ERP", tested OK over both
  WiFi and Ethernet, with a note that it is not reachable from home.
- AS400 keeps its own area, "AS400 / IBM i", still pending test.
- Title banners no longer present SAP E01 as the project scope.
- 18 systems instead of 17; all dashboard totals reconcile.

Also rewrote the instructions, notes and labels in plainer language,
shortened the column headers, and dropped the observations that merely
restated the status columns.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WqMtBjpHrU1DDNujKeeug7
</commit_message>
<xml_diff>
--- a/tracking/SAP_E01_Seguimiento_Pruebas_Accesos.xlsx
+++ b/tracking/SAP_E01_Seguimiento_Pruebas_Accesos.xlsx
@@ -14,10 +14,10 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">Listas!$A$1:$F$13</definedName>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Resumen!$A$1:$Q$53</definedName>
-    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">Seguimiento!$A$1:$N$44</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Resumen!$A$1:$Q$52</definedName>
+    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">Seguimiento!$A$1:$N$45</definedName>
     <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Titles" vbProcedure="false">Seguimiento!$1:$6</definedName>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Seguimiento!$A$6:$N$33</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Seguimiento!$A$6:$N$34</definedName>
     <definedName function="false" hidden="false" name="lst_Accion" vbProcedure="false">Listas!$C$6:$C$13</definedName>
     <definedName function="false" hidden="false" name="lst_Conexion" vbProcedure="false">Listas!$D$6:$D$9</definedName>
     <definedName function="false" hidden="false" name="lst_Criticidad" vbProcedure="false">Listas!$E$6:$E$9</definedName>
@@ -46,12 +46,11 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Columna calculada — no la edite.
-Acceso total (WiFi + Cable): WiFi = OK y Cable = OK
-Solo WiFi: WiFi = OK y Cable distinto de OK
-Solo cable Ethernet: Cable = OK y WiFi distinto de OK
-Sin acceso: WiFi = KO y Cable = KO
-Pendiente: cualquier otra combinación</t>
+          <t xml:space="preserve">Se calcula solo, no editar.
+WiFi OK + cable OK  -&gt;  WiFi y cable
+Solo uno de los dos OK  -&gt;  Solo WiFi / Solo cable
+Los dos KO  -&gt;  Sin acceso
+Resto  -&gt;  Pendiente</t>
         </r>
       </text>
     </comment>
@@ -63,8 +62,29 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">La criticidad precargada es una PROPUESTA INICIAL: no venía en el listado de origen.
-Ajústela según el impacto real en el negocio.</t>
+          <t xml:space="preserve">Estimación propia, no venía en el listado original. Revisar.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <authors>
+    <author>Unknown Author</author>
+  </authors>
+  <commentList>
+    <comment ref="F5" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Esta columna es informativa: el resultado se calcula en la hoja Seguimiento.</t>
         </r>
       </text>
     </comment>
@@ -73,60 +93,51 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="147">
-  <si>
-    <t xml:space="preserve">PANEL DE CONTROL — PRUEBAS DE ACCESO A SISTEMAS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SAP E01  ·  Todos los indicadores se calculan a partir de la hoja «Seguimiento» y se actualizan solos al editarla</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SISTEMAS EN SEGUIMIENTO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">YA PROBADOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PENDIENTES DE PROBAR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">% DE AVANCE DE LAS PRUEBAS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ACCESO TOTAL (WIFI + CABLE)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ACCESO LIMITADO (UN SOLO MEDIO)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SIN ACCESO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CRÍTICOS SIN ACCESO COMPLETO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DISTRIBUCIÓN POR RESULTADO DE CONECTIVIDAD</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="139">
+  <si>
+    <t xml:space="preserve">RESUMEN DE PRUEBAS DE ACCESO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se actualiza solo a partir de la hoja Seguimiento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sistemas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Probados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pendientes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% probado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WiFi y cable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solo un medio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sin acceso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Críticos sin acceso completo</t>
   </si>
   <si>
     <t xml:space="preserve">Resultado de conectividad</t>
   </si>
   <si>
-    <t xml:space="preserve">Sistemas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">% del total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Acceso total (WiFi + Cable)</t>
+    <t xml:space="preserve">Resultado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">%</t>
   </si>
   <si>
     <t xml:space="preserve">Solo WiFi</t>
   </si>
   <si>
-    <t xml:space="preserve">Solo cable Ethernet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sin acceso</t>
+    <t xml:space="preserve">Solo cable</t>
   </si>
   <si>
     <t xml:space="preserve">Pendiente</t>
@@ -138,19 +149,16 @@
     <t xml:space="preserve">TOTAL</t>
   </si>
   <si>
-    <t xml:space="preserve">DISTRIBUCIÓN POR ÁREA FUNCIONAL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Área funcional</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Acceso total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Acceso limitado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SAP E01 / ERP</t>
+    <t xml:space="preserve">Por área</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Área</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SAP / ERP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AS400 / IBM i</t>
   </si>
   <si>
     <t xml:space="preserve">WITRON / CPMS</t>
@@ -171,13 +179,13 @@
     <t xml:space="preserve">Escritorio remoto</t>
   </si>
   <si>
-    <t xml:space="preserve">PRÓXIMAS ACCIONES</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Próxima acción</t>
-  </si>
-  <si>
-    <t xml:space="preserve">De los cuales, críticos o de prioridad alta</t>
+    <t xml:space="preserve">Siguientes pasos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Siguiente paso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">De ellos, críticos o de prioridad alta</t>
   </si>
   <si>
     <t xml:space="preserve">Ninguna</t>
@@ -186,46 +194,46 @@
     <t xml:space="preserve">Programar prueba</t>
   </si>
   <si>
-    <t xml:space="preserve">Instalar / Configurar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Solicitar acceso a IT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Escalar a IT / Redes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Revisar VPN / Firewall</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reprogramar prueba</t>
+    <t xml:space="preserve">Instalar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pedir acceso a IT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Escalar a Redes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revisar VPN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Repetir prueba</t>
   </si>
   <si>
     <t xml:space="preserve">En seguimiento</t>
   </si>
   <si>
-    <t xml:space="preserve">•   Fuente: listado «SAP E01 – Pendiente de prueba» facilitado por el usuario. Los resultados de WiFi y de cable Ethernet reproducen literalmente ese listado.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">•   La columna «Criticidad» de la hoja «Seguimiento» es una propuesta inicial y no venía en el listado de origen: revísela antes de usarla para priorizar.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">•   Ningún indicador de esta hoja está escrito a mano: todos son fórmulas COUNTIF/COUNTIFS sobre la hoja «Seguimiento» (filas 7 a 33, con margen para dar de alta sistemas nuevos).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SEGUIMIENTO DE PRUEBAS DE ACCESO A SISTEMAS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SAP E01  ·  Validación de conectividad desde la red de DS Smith  —  WiFi vs. cable Ethernet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CÓMO USAR ESTA HOJA:   rellene únicamente las celdas de fondo crema — «Estado de la prueba», «WiFi», «Cable Ethernet», «Criticidad», «Responsable», «Fecha de prueba», «Próxima acción» y «Observaciones» —, todas ellas con desplegable salvo las de texto libre y la fecha.   La columna «Resultado de conectividad» se calcula sola y no debe editarse.   Las filas vacías del final están listas para añadir sistemas nuevos: se contabilizan solas en la hoja «Resumen».</t>
-  </si>
-  <si>
-    <t xml:space="preserve">■  Acceso total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">■  Solo WiFi / solo cable</t>
+    <t xml:space="preserve">•   Datos del listado de pruebas original.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">•   La criticidad es una estimación, no venía en el listado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">•   Todos los números salen de la hoja Seguimiento, filas 7 a 34.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRUEBAS DE ACCESO A SISTEMAS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conectividad desde la red de DS Smith: WiFi y cable Ethernet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Las celdas en crema se rellenan a mano, casi todas con desplegable. La columna Resultado se calcula sola, no tocar. Las filas vacías del final son para dar de alta sistemas nuevos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">■  WiFi y cable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">■  Solo un medio</t>
   </si>
   <si>
     <t xml:space="preserve">■  Sin acceso</t>
@@ -237,28 +245,28 @@
     <t xml:space="preserve">■  En curso</t>
   </si>
   <si>
-    <t xml:space="preserve">■  Celdas a rellenar (fondo crema)</t>
+    <t xml:space="preserve">■  Se rellena a mano</t>
   </si>
   <si>
     <t xml:space="preserve">N.º</t>
   </si>
   <si>
-    <t xml:space="preserve">Sistema / Aplicación</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ámbito geográfico</t>
-  </si>
-  <si>
-    <t xml:space="preserve">URL / Vía de acceso</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estado de la prueba</t>
+    <t xml:space="preserve">Sistema</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ámbito</t>
+  </si>
+  <si>
+    <t xml:space="preserve">URL / Acceso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estado</t>
   </si>
   <si>
     <t xml:space="preserve">WiFi</t>
   </si>
   <si>
-    <t xml:space="preserve">Cable Ethernet</t>
+    <t xml:space="preserve">Cable</t>
   </si>
   <si>
     <t xml:space="preserve">Criticidad</t>
@@ -267,12 +275,27 @@
     <t xml:space="preserve">Responsable</t>
   </si>
   <si>
-    <t xml:space="preserve">Fecha de prueba</t>
+    <t xml:space="preserve">Fecha</t>
   </si>
   <si>
     <t xml:space="preserve">Observaciones</t>
   </si>
   <si>
+    <t xml:space="preserve">SAP E01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Probado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crítica</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No accesible desde casa. Solo desde la red de DS Smith.</t>
+  </si>
+  <si>
     <t xml:space="preserve">AS400</t>
   </si>
   <si>
@@ -288,10 +311,7 @@
     <t xml:space="preserve">No probado</t>
   </si>
   <si>
-    <t xml:space="preserve">Crítica</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pendiente de probar en las tres geografías (España, Francia e Italia).</t>
+    <t xml:space="preserve">Falta probarlo en las tres geografías.</t>
   </si>
   <si>
     <t xml:space="preserve">Citrix — acceso a WITRON</t>
@@ -303,16 +323,10 @@
     <t xml:space="preserve">https://ipstorefront.ipaper.com/</t>
   </si>
   <si>
-    <t xml:space="preserve">Probado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OK</t>
-  </si>
-  <si>
     <t xml:space="preserve">KO</t>
   </si>
   <si>
-    <t xml:space="preserve">Probado con éxito mediante WiFi. Por cable Ethernet no funciona (WITRON/CPMS — España).</t>
+    <t xml:space="preserve">Por WiFi bien; por cable no funciona (WITRON/CPMS España).</t>
   </si>
   <si>
     <t xml:space="preserve">Sage — acceso a Adonix (CARPA)</t>
@@ -327,7 +341,7 @@
     <t xml:space="preserve">Alta</t>
   </si>
   <si>
-    <t xml:space="preserve">Sin acceso desde la red de DS Smith, ni por WiFi ni por cable. En el listado original aparecía duplicado (bloques 1 y 2) con el mismo resultado; se ha consolidado en esta única fila.</t>
+    <t xml:space="preserve">Venía duplicado en el listado original.</t>
   </si>
   <si>
     <t xml:space="preserve">SharePoint / OneDrive IP</t>
@@ -342,9 +356,6 @@
     <t xml:space="preserve">Media</t>
   </si>
   <si>
-    <t xml:space="preserve">Probado con éxito mediante WiFi y cable Ethernet.</t>
-  </si>
-  <si>
     <t xml:space="preserve">DMT Tool</t>
   </si>
   <si>
@@ -360,25 +371,25 @@
     <t xml:space="preserve">https://miacceso.e-factura.net/</t>
   </si>
   <si>
-    <t xml:space="preserve">Acceso remoto a RSVGEST (escritorio)</t>
+    <t xml:space="preserve">Acceso remoto a RSVGEST</t>
   </si>
   <si>
     <t xml:space="preserve">España (Tavernes Madera)</t>
   </si>
   <si>
-    <t xml:space="preserve">Escritorio remoto al PC de Tavernes Madera</t>
+    <t xml:space="preserve">Escritorio remoto al PC de Tavernes</t>
   </si>
   <si>
     <t xml:space="preserve">Pendiente de instalación</t>
   </si>
   <si>
-    <t xml:space="preserve">Pendiente de instalación para poder probarlo.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gestión PDF — descarga de facturas SERES</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aplicación de escritorio (descarga de PDF desde SERES)</t>
+    <t xml:space="preserve">Falta instalarlo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gestión PDF (facturas SERES)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aplicación de escritorio</t>
   </si>
   <si>
     <t xml:space="preserve">My Access</t>
@@ -396,18 +407,12 @@
     <t xml:space="preserve">https://ocr.emea.ipaper.com/</t>
   </si>
   <si>
-    <t xml:space="preserve">Sin acceso ni por WiFi ni por cable.</t>
-  </si>
-  <si>
     <t xml:space="preserve">ECM</t>
   </si>
   <si>
     <t xml:space="preserve">https://ecm.emea.ipaper.com/</t>
   </si>
   <si>
-    <t xml:space="preserve">Con acceso tanto por WiFi como por cable.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Xelix</t>
   </si>
   <si>
@@ -417,10 +422,7 @@
     <t xml:space="preserve">Accounts Payable (Matchpay)</t>
   </si>
   <si>
-    <t xml:space="preserve">URL no facilitada en el listado original</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sin acceso ni por WiFi ni por cable. Falta confirmar la URL de acceso.</t>
+    <t xml:space="preserve">Falta la URL.</t>
   </si>
   <si>
     <t xml:space="preserve">AP Upload (Matchpay)</t>
@@ -429,7 +431,7 @@
     <t xml:space="preserve">https://apupload.ipaper.com/</t>
   </si>
   <si>
-    <t xml:space="preserve">BI iPaper — informes Matchpay</t>
+    <t xml:space="preserve">BI iPaper (informes Matchpay)</t>
   </si>
   <si>
     <t xml:space="preserve">https://bi.ipaper.com/BOE/BI/logonNoSso.jsp</t>
@@ -444,19 +446,16 @@
     <t xml:space="preserve">http://s02afnbgp03.na.ipaper.com/P8LoadViewer/</t>
   </si>
   <si>
-    <t xml:space="preserve">Sin acceso ni por WiFi ni por cable. La URL completa del listado original incluye el parámetro ?TeamsCID=c00c9452-e557-4935-b77a-43fc65957a5b.</t>
+    <t xml:space="preserve">URL completa con ?TeamsCID=c00c9452-e557-4935-b77a-43fc65957a5b</t>
   </si>
   <si>
     <t xml:space="preserve">Arrows (CARPA)</t>
   </si>
   <si>
-    <t xml:space="preserve">Acceso mediante escritorio remoto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FILA DE EJEMPLO — muestra el formato esperado al dar de alta un sistema nuevo. No se contabiliza en la hoja «Resumen»; escriba los sistemas nuevos en las filas libres de la tabla de arriba.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18</t>
+    <t xml:space="preserve">Ejemplo de cómo rellenar una fila. No cuenta en el Resumen; los sistemas nuevos van en las filas vacías de arriba.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19</t>
   </si>
   <si>
     <t xml:space="preserve">Nombre del sistema</t>
@@ -471,40 +470,37 @@
     <t xml:space="preserve">12/08/2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Acceso correcto por WiFi; por cable Ethernet devuelve tiempo de espera agotado.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOTAS Y SUPUESTOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">•   Fuente de los datos: listado «SAP E01 – Pendiente de prueba» facilitado por el usuario. Los estados y resultados de WiFi/cable reproducen literalmente ese listado.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">•   «Criticidad»: propuesta inicial elaborada al construir este libro; NO figuraba en el listado de origen. Revísela y ajústela.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">•   «Sage — acceso a Adonix (CARPA)» aparecía dos veces en el listado de origen (bloques 1 y 2) con idéntico resultado: se ha consolidado en una sola fila (N.º 3). Por eso el libro recoge 17 sistemas y no 18.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">•   «Accounts Payable (Matchpay)» no traía URL en el listado de origen; queda pendiente de confirmar.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">•   «Responsable» y «Fecha de prueba» se dejan en blanco a propósito, para que los complete quien realice las pruebas.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">•   Todo lo que se escriba en las filas libres de la tabla se suma automáticamente a los indicadores de la hoja «Resumen».</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LISTAS DE VALORES DE LOS DESPLEGABLES</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puede añadir o modificar valores en estas columnas: los desplegables de la hoja «Seguimiento» se actualizan automáticamente. No borre las cabeceras.</t>
+    <t xml:space="preserve">Por WiFi entra; por cable da tiempo de espera agotado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOTAS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">•   Los resultados de WiFi y cable vienen del listado de pruebas original.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">•   SAP E01 y AS400 son sistemas distintos, cada uno en su fila.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">•   Falta el ámbito geográfico de SAP E01 y la URL de Accounts Payable (Matchpay).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">•   La criticidad es una estimación, no venía en el listado. Conviene revisarla.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">•   Sage/Adonix venía duplicado en el listado, con el mismo resultado las dos veces. Se ha unificado en la fila 4, por eso salen 18 sistemas y no 19.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">•   Responsable y fecha se han dejado en blanco para rellenarlos según se vaya probando.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VALORES DE LOS DESPLEGABLES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se pueden añadir o cambiar valores. Los desplegables de Seguimiento se actualizan solos. No borrar las cabeceras.</t>
   </si>
   <si>
     <t xml:space="preserve">WiFi / Cable</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resultado (calculado)</t>
   </si>
   <si>
     <t xml:space="preserve">En curso</t>
@@ -592,7 +588,7 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="8"/>
+      <sz val="9"/>
       <color rgb="FF6B7683"/>
       <name val="Arial"/>
       <family val="0"/>
@@ -1092,7 +1088,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="86">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1261,80 +1257,88 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="10" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="14" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="33" fillId="14" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="32" fillId="11" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="11" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="11" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="11" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="34" fillId="10" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="34" fillId="11" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="21" fillId="10" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="32" fillId="11" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="10" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="14" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="33" fillId="14" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="11" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="32" fillId="11" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="11" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="11" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="21" fillId="11" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="34" fillId="11" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="11" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="34" fillId="10" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="21" fillId="11" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="10" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="10" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="10" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="21" fillId="10" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="14" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="10" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="20" fillId="11" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="14" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -1349,20 +1353,24 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="32" fillId="10" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="32" fillId="11" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="10" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="14" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="10" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="20" fillId="11" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="14" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -1389,8 +1397,12 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="21" fillId="15" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="36" fillId="7" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="21" fillId="15" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -2037,13 +2049,13 @@
               <c:strCache>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>Acceso total (WiFi + Cable)</c:v>
+                  <c:v>WiFi y cable</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>Solo WiFi</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Solo cable Ethernet</c:v>
+                  <c:v>Solo cable</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>Sin acceso</c:v>
@@ -2064,7 +2076,7 @@
                 <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>6</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>1</c:v>
@@ -2161,7 +2173,7 @@
                 </a:solidFill>
                 <a:latin typeface="Calibri"/>
               </a:rPr>
-              <a:t>Situación por área funcional</a:t>
+              <a:t>Por área</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -2189,7 +2201,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Acceso total</c:v>
+                  <c:v>WiFi y cable</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2232,28 +2244,31 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Resumen!$B$26:$B$32</c:f>
+              <c:f>Resumen!$B$26:$B$33</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>SAP E01 / ERP</c:v>
+                  <c:v>SAP / ERP</c:v>
                 </c:pt>
                 <c:pt idx="1">
+                  <c:v>AS400 / IBM i</c:v>
+                </c:pt>
+                <c:pt idx="2">
                   <c:v>WITRON / CPMS</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>CARPA</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>Cuentas a pagar (Matchpay)</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>Facturación electrónica</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="6">
                   <c:v>Ofimática y colaboración</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="7">
                   <c:v>Escritorio remoto</c:v>
                 </c:pt>
               </c:strCache>
@@ -2261,12 +2276,12 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Resumen!$F$26:$F$32</c:f>
+              <c:f>Resumen!$F$26:$F$33</c:f>
               <c:numCache>
                 <c:formatCode>#,##0;;\–</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -2275,15 +2290,18 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>2</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>1</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="6">
                   <c:v>3</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="7">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -2299,7 +2317,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Acceso limitado</c:v>
+                  <c:v>Solo un medio</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2342,28 +2360,31 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Resumen!$B$26:$B$32</c:f>
+              <c:f>Resumen!$B$26:$B$33</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>SAP E01 / ERP</c:v>
+                  <c:v>SAP / ERP</c:v>
                 </c:pt>
                 <c:pt idx="1">
+                  <c:v>AS400 / IBM i</c:v>
+                </c:pt>
+                <c:pt idx="2">
                   <c:v>WITRON / CPMS</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>CARPA</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>Cuentas a pagar (Matchpay)</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>Facturación electrónica</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="6">
                   <c:v>Ofimática y colaboración</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="7">
                   <c:v>Escritorio remoto</c:v>
                 </c:pt>
               </c:strCache>
@@ -2371,18 +2392,18 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Resumen!$G$26:$G$32</c:f>
+              <c:f>Resumen!$G$26:$G$33</c:f>
               <c:numCache>
                 <c:formatCode>#,##0;;\–</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
                   <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -2394,6 +2415,9 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="6">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="7">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -2452,28 +2476,31 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Resumen!$B$26:$B$32</c:f>
+              <c:f>Resumen!$B$26:$B$33</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>SAP E01 / ERP</c:v>
+                  <c:v>SAP / ERP</c:v>
                 </c:pt>
                 <c:pt idx="1">
+                  <c:v>AS400 / IBM i</c:v>
+                </c:pt>
+                <c:pt idx="2">
                   <c:v>WITRON / CPMS</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>CARPA</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>Cuentas a pagar (Matchpay)</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>Facturación electrónica</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="6">
                   <c:v>Ofimática y colaboración</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="7">
                   <c:v>Escritorio remoto</c:v>
                 </c:pt>
               </c:strCache>
@@ -2481,10 +2508,10 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Resumen!$H$26:$H$32</c:f>
+              <c:f>Resumen!$H$26:$H$33</c:f>
               <c:numCache>
                 <c:formatCode>#,##0;;\–</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -2492,18 +2519,21 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
                   <c:v>2</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>5</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="6">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="7">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -2562,28 +2592,31 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Resumen!$B$26:$B$32</c:f>
+              <c:f>Resumen!$B$26:$B$33</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>SAP E01 / ERP</c:v>
+                  <c:v>SAP / ERP</c:v>
                 </c:pt>
                 <c:pt idx="1">
+                  <c:v>AS400 / IBM i</c:v>
+                </c:pt>
+                <c:pt idx="2">
                   <c:v>WITRON / CPMS</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>CARPA</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>Cuentas a pagar (Matchpay)</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>Facturación electrónica</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="6">
                   <c:v>Ofimática y colaboración</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="7">
                   <c:v>Escritorio remoto</c:v>
                 </c:pt>
               </c:strCache>
@@ -2591,15 +2624,15 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Resumen!$I$26:$I$32</c:f>
+              <c:f>Resumen!$I$26:$I$33</c:f>
               <c:numCache>
                 <c:formatCode>#,##0;;\–</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="8"/>
                 <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2608,12 +2641,15 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="5">
                   <c:v>1</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="6">
                   <c:v>0</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="7">
                   <c:v>1</c:v>
                 </c:pt>
               </c:numCache>
@@ -2622,11 +2658,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="4973886"/>
-        <c:axId val="38603313"/>
+        <c:axId val="26935589"/>
+        <c:axId val="49265764"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="4973886"/>
+        <c:axId val="26935589"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2658,7 +2694,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="38603313"/>
+        <c:crossAx val="49265764"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2666,7 +2702,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="38603313"/>
+        <c:axId val="49265764"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2698,7 +2734,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="4973886"/>
+        <c:crossAx val="26935589"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2763,7 +2799,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>67320</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>55800</xdr:rowOff>
+      <xdr:rowOff>75240</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2771,7 +2807,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="7154640" y="3105000"/>
+        <a:off x="7154640" y="3048120"/>
         <a:ext cx="4895640" cy="2951640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -2793,7 +2829,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>67320</xdr:colOff>
       <xdr:row>35</xdr:row>
-      <xdr:rowOff>151560</xdr:rowOff>
+      <xdr:rowOff>113040</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2801,7 +2837,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="7154640" y="6496200"/>
+        <a:off x="7154640" y="6419880"/>
         <a:ext cx="4895640" cy="2951640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -3053,31 +3089,31 @@
     <row r="3" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="4" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="n">
-        <f aca="false">COUNTA(Seguimiento!$B$7:$B$33)</f>
-        <v>17</v>
+        <f aca="false">COUNTA(Seguimiento!$B$7:$B$34)</f>
+        <v>18</v>
       </c>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
       <c r="F4" s="4" t="n">
-        <f aca="false">COUNTIF(Seguimiento!$F$7:$F$33,"Probado")</f>
-        <v>14</v>
+        <f aca="false">COUNTIF(Seguimiento!$F$7:$F$34,"Probado")</f>
+        <v>15</v>
       </c>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
       <c r="J4" s="5" t="n">
-        <f aca="false">COUNTA(Seguimiento!$B$7:$B$33)-COUNTIF(Seguimiento!$F$7:$F$33,"Probado")-COUNTIF(Seguimiento!$F$7:$F$33,"No aplica")</f>
+        <f aca="false">COUNTA(Seguimiento!$B$7:$B$34)-COUNTIF(Seguimiento!$F$7:$F$34,"Probado")-COUNTIF(Seguimiento!$F$7:$F$34,"No aplica")</f>
         <v>3</v>
       </c>
       <c r="K4" s="5"/>
       <c r="L4" s="5"/>
       <c r="N4" s="6" t="n">
-        <f aca="false">IFERROR(COUNTIF(Seguimiento!$F$7:$F$33,"Probado")/MAX(1,COUNTA(Seguimiento!$B$7:$B$33)-COUNTIF(Seguimiento!$F$7:$F$33,"No aplica")),0)</f>
-        <v>0.823529411764706</v>
+        <f aca="false">IFERROR(COUNTIF(Seguimiento!$F$7:$F$34,"Probado")/MAX(1,COUNTA(Seguimiento!$B$7:$B$34)-COUNTIF(Seguimiento!$F$7:$F$34,"No aplica")),0)</f>
+        <v>0.833333333333333</v>
       </c>
       <c r="O4" s="6"/>
       <c r="P4" s="6"/>
     </row>
-    <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="7" t="s">
         <v>2</v>
       </c>
@@ -3102,31 +3138,31 @@
     <row r="6" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="7" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="4" t="n">
-        <f aca="false">COUNTIF(Seguimiento!$I$7:$I$33,"Acceso total (WiFi + Cable)")</f>
-        <v>6</v>
+        <f aca="false">COUNTIF(Seguimiento!$I$7:$I$34,"WiFi y cable")</f>
+        <v>7</v>
       </c>
       <c r="C7" s="4"/>
       <c r="D7" s="4"/>
       <c r="F7" s="5" t="n">
-        <f aca="false">COUNTIF(Seguimiento!$I$7:$I$33,"Solo WiFi")+COUNTIF(Seguimiento!$I$7:$I$33,"Solo cable Ethernet")</f>
+        <f aca="false">COUNTIF(Seguimiento!$I$7:$I$34,"Solo WiFi")+COUNTIF(Seguimiento!$I$7:$I$34,"Solo cable")</f>
         <v>1</v>
       </c>
       <c r="G7" s="5"/>
       <c r="H7" s="5"/>
       <c r="J7" s="8" t="n">
-        <f aca="false">COUNTIF(Seguimiento!$I$7:$I$33,"Sin acceso")</f>
+        <f aca="false">COUNTIF(Seguimiento!$I$7:$I$34,"Sin acceso")</f>
         <v>7</v>
       </c>
       <c r="K7" s="8"/>
       <c r="L7" s="8"/>
       <c r="N7" s="8" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$J$7:$J$33,"Crítica",Seguimiento!$I$7:$I$33,"&lt;&gt;Acceso total (WiFi + Cable)",Seguimiento!$B$7:$B$33,"&lt;&gt;")</f>
+        <f aca="false">COUNTIFS(Seguimiento!$J$7:$J$34,"Crítica",Seguimiento!$I$7:$I$34,"&lt;&gt;WiFi y cable",Seguimiento!$B$7:$B$34,"&lt;&gt;")</f>
         <v>2</v>
       </c>
       <c r="O7" s="8"/>
       <c r="P7" s="8"/>
     </row>
-    <row r="8" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="7" t="s">
         <v>6</v>
       </c>
@@ -3169,57 +3205,57 @@
       <c r="P10" s="9"/>
       <c r="Q10" s="9"/>
     </row>
-    <row r="11" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="10" t="s">
         <v>11</v>
       </c>
       <c r="C11" s="10"/>
       <c r="D11" s="10"/>
       <c r="E11" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="F11" s="11" t="s">
         <v>12</v>
-      </c>
-      <c r="F11" s="11" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="12" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C12" s="12"/>
       <c r="D12" s="12"/>
       <c r="E12" s="13" t="n">
-        <f aca="false">COUNTIF(Seguimiento!$I$7:$I$33,$B12)</f>
-        <v>6</v>
+        <f aca="false">COUNTIF(Seguimiento!$I$7:$I$34,$B12)</f>
+        <v>7</v>
       </c>
       <c r="F12" s="14" t="n">
         <f aca="false">IFERROR($E12/$E$18,0)</f>
-        <v>0.352941176470588</v>
+        <v>0.388888888888889</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="15" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C13" s="15"/>
       <c r="D13" s="15"/>
       <c r="E13" s="13" t="n">
-        <f aca="false">COUNTIF(Seguimiento!$I$7:$I$33,$B13)</f>
+        <f aca="false">COUNTIF(Seguimiento!$I$7:$I$34,$B13)</f>
         <v>1</v>
       </c>
       <c r="F13" s="14" t="n">
         <f aca="false">IFERROR($E13/$E$18,0)</f>
-        <v>0.0588235294117647</v>
+        <v>0.0555555555555556</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="15" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C14" s="15"/>
       <c r="D14" s="15"/>
       <c r="E14" s="13" t="n">
-        <f aca="false">COUNTIF(Seguimiento!$I$7:$I$33,$B14)</f>
+        <f aca="false">COUNTIF(Seguimiento!$I$7:$I$34,$B14)</f>
         <v>0</v>
       </c>
       <c r="F14" s="14" t="n">
@@ -3229,42 +3265,42 @@
     </row>
     <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="16" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="C15" s="16"/>
       <c r="D15" s="16"/>
       <c r="E15" s="13" t="n">
-        <f aca="false">COUNTIF(Seguimiento!$I$7:$I$33,$B15)</f>
+        <f aca="false">COUNTIF(Seguimiento!$I$7:$I$34,$B15)</f>
         <v>7</v>
       </c>
       <c r="F15" s="14" t="n">
         <f aca="false">IFERROR($E15/$E$18,0)</f>
-        <v>0.411764705882353</v>
+        <v>0.388888888888889</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="17" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C16" s="17"/>
       <c r="D16" s="17"/>
       <c r="E16" s="13" t="n">
-        <f aca="false">COUNTIF(Seguimiento!$I$7:$I$33,$B16)</f>
+        <f aca="false">COUNTIF(Seguimiento!$I$7:$I$34,$B16)</f>
         <v>3</v>
       </c>
       <c r="F16" s="14" t="n">
         <f aca="false">IFERROR($E16/$E$18,0)</f>
-        <v>0.176470588235294</v>
+        <v>0.166666666666667</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="17" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C17" s="17"/>
       <c r="D17" s="17"/>
       <c r="E17" s="13" t="n">
-        <f aca="false">COUNTIF(Seguimiento!$I$7:$I$33,$B17)</f>
+        <f aca="false">COUNTIF(Seguimiento!$I$7:$I$34,$B17)</f>
         <v>0</v>
       </c>
       <c r="F17" s="14" t="n">
@@ -3274,13 +3310,13 @@
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="18" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C18" s="18"/>
       <c r="D18" s="18"/>
       <c r="E18" s="19" t="n">
         <f aca="false">SUM(E12:E17)</f>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F18" s="20" t="n">
         <f aca="false">IFERROR($E18/$E18,0)</f>
@@ -3289,7 +3325,7 @@
     </row>
     <row r="24" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="9" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="C24" s="9"/>
       <c r="D24" s="9"/>
@@ -3307,260 +3343,287 @@
       <c r="P24" s="9"/>
       <c r="Q24" s="9"/>
     </row>
-    <row r="25" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="10" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C25" s="10"/>
       <c r="D25" s="10"/>
       <c r="E25" s="11" t="s">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="G25" s="11" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="H25" s="11" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="I25" s="11" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="21" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="C26" s="21"/>
       <c r="D26" s="21"/>
       <c r="E26" s="22" t="n">
-        <f aca="false">COUNTIF(Seguimiento!$C$7:$C$33,$B26)</f>
+        <f aca="false">COUNTIF(Seguimiento!$C$7:$C$34,$B26)</f>
         <v>1</v>
       </c>
       <c r="F26" s="23" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$33,$B26,Seguimiento!$I$7:$I$33,"Acceso total (WiFi + Cable)")</f>
+        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$34,$B26,Seguimiento!$I$7:$I$34,"WiFi y cable")</f>
+        <v>1</v>
+      </c>
+      <c r="G26" s="23" t="n">
+        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$34,$B26,Seguimiento!$I$7:$I$34,"Solo WiFi")+COUNTIFS(Seguimiento!$C$7:$C$34,$B26,Seguimiento!$I$7:$I$34,"Solo cable")</f>
         <v>0</v>
       </c>
-      <c r="G26" s="23" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$33,$B26,Seguimiento!$I$7:$I$33,"Solo WiFi")+COUNTIFS(Seguimiento!$C$7:$C$33,$B26,Seguimiento!$I$7:$I$33,"Solo cable Ethernet")</f>
+      <c r="H26" s="23" t="n">
+        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$34,$B26,Seguimiento!$I$7:$I$34,"Sin acceso")</f>
         <v>0</v>
       </c>
-      <c r="H26" s="23" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$33,$B26,Seguimiento!$I$7:$I$33,"Sin acceso")</f>
+      <c r="I26" s="23" t="n">
+        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$34,$B26,Seguimiento!$I$7:$I$34,"Pendiente")</f>
         <v>0</v>
-      </c>
-      <c r="I26" s="23" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$33,$B26,Seguimiento!$I$7:$I$33,"Pendiente")</f>
-        <v>1</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="24" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C27" s="24"/>
       <c r="D27" s="24"/>
       <c r="E27" s="25" t="n">
-        <f aca="false">COUNTIF(Seguimiento!$C$7:$C$33,$B27)</f>
+        <f aca="false">COUNTIF(Seguimiento!$C$7:$C$34,$B27)</f>
         <v>1</v>
       </c>
       <c r="F27" s="26" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$33,$B27,Seguimiento!$I$7:$I$33,"Acceso total (WiFi + Cable)")</f>
+        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$34,$B27,Seguimiento!$I$7:$I$34,"WiFi y cable")</f>
         <v>0</v>
       </c>
       <c r="G27" s="26" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$33,$B27,Seguimiento!$I$7:$I$33,"Solo WiFi")+COUNTIFS(Seguimiento!$C$7:$C$33,$B27,Seguimiento!$I$7:$I$33,"Solo cable Ethernet")</f>
+        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$34,$B27,Seguimiento!$I$7:$I$34,"Solo WiFi")+COUNTIFS(Seguimiento!$C$7:$C$34,$B27,Seguimiento!$I$7:$I$34,"Solo cable")</f>
+        <v>0</v>
+      </c>
+      <c r="H27" s="26" t="n">
+        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$34,$B27,Seguimiento!$I$7:$I$34,"Sin acceso")</f>
+        <v>0</v>
+      </c>
+      <c r="I27" s="26" t="n">
+        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$34,$B27,Seguimiento!$I$7:$I$34,"Pendiente")</f>
         <v>1</v>
-      </c>
-      <c r="H27" s="26" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$33,$B27,Seguimiento!$I$7:$I$33,"Sin acceso")</f>
-        <v>0</v>
-      </c>
-      <c r="I27" s="26" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$33,$B27,Seguimiento!$I$7:$I$33,"Pendiente")</f>
-        <v>0</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="21" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="C28" s="21"/>
       <c r="D28" s="21"/>
       <c r="E28" s="22" t="n">
-        <f aca="false">COUNTIF(Seguimiento!$C$7:$C$33,$B28)</f>
-        <v>2</v>
+        <f aca="false">COUNTIF(Seguimiento!$C$7:$C$34,$B28)</f>
+        <v>1</v>
       </c>
       <c r="F28" s="23" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$33,$B28,Seguimiento!$I$7:$I$33,"Acceso total (WiFi + Cable)")</f>
+        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$34,$B28,Seguimiento!$I$7:$I$34,"WiFi y cable")</f>
         <v>0</v>
       </c>
       <c r="G28" s="23" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$33,$B28,Seguimiento!$I$7:$I$33,"Solo WiFi")+COUNTIFS(Seguimiento!$C$7:$C$33,$B28,Seguimiento!$I$7:$I$33,"Solo cable Ethernet")</f>
+        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$34,$B28,Seguimiento!$I$7:$I$34,"Solo WiFi")+COUNTIFS(Seguimiento!$C$7:$C$34,$B28,Seguimiento!$I$7:$I$34,"Solo cable")</f>
+        <v>1</v>
+      </c>
+      <c r="H28" s="23" t="n">
+        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$34,$B28,Seguimiento!$I$7:$I$34,"Sin acceso")</f>
         <v>0</v>
       </c>
-      <c r="H28" s="23" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$33,$B28,Seguimiento!$I$7:$I$33,"Sin acceso")</f>
-        <v>2</v>
-      </c>
       <c r="I28" s="23" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$33,$B28,Seguimiento!$I$7:$I$33,"Pendiente")</f>
+        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$34,$B28,Seguimiento!$I$7:$I$34,"Pendiente")</f>
         <v>0</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B29" s="24" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="C29" s="24"/>
       <c r="D29" s="24"/>
       <c r="E29" s="25" t="n">
-        <f aca="false">COUNTIF(Seguimiento!$C$7:$C$33,$B29)</f>
-        <v>7</v>
+        <f aca="false">COUNTIF(Seguimiento!$C$7:$C$34,$B29)</f>
+        <v>2</v>
       </c>
       <c r="F29" s="26" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$33,$B29,Seguimiento!$I$7:$I$33,"Acceso total (WiFi + Cable)")</f>
+        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$34,$B29,Seguimiento!$I$7:$I$34,"WiFi y cable")</f>
+        <v>0</v>
+      </c>
+      <c r="G29" s="26" t="n">
+        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$34,$B29,Seguimiento!$I$7:$I$34,"Solo WiFi")+COUNTIFS(Seguimiento!$C$7:$C$34,$B29,Seguimiento!$I$7:$I$34,"Solo cable")</f>
+        <v>0</v>
+      </c>
+      <c r="H29" s="26" t="n">
+        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$34,$B29,Seguimiento!$I$7:$I$34,"Sin acceso")</f>
         <v>2</v>
       </c>
-      <c r="G29" s="26" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$33,$B29,Seguimiento!$I$7:$I$33,"Solo WiFi")+COUNTIFS(Seguimiento!$C$7:$C$33,$B29,Seguimiento!$I$7:$I$33,"Solo cable Ethernet")</f>
-        <v>0</v>
-      </c>
-      <c r="H29" s="26" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$33,$B29,Seguimiento!$I$7:$I$33,"Sin acceso")</f>
-        <v>5</v>
-      </c>
       <c r="I29" s="26" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$33,$B29,Seguimiento!$I$7:$I$33,"Pendiente")</f>
+        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$34,$B29,Seguimiento!$I$7:$I$34,"Pendiente")</f>
         <v>0</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="21" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="C30" s="21"/>
       <c r="D30" s="21"/>
       <c r="E30" s="22" t="n">
-        <f aca="false">COUNTIF(Seguimiento!$C$7:$C$33,$B30)</f>
+        <f aca="false">COUNTIF(Seguimiento!$C$7:$C$34,$B30)</f>
+        <v>7</v>
+      </c>
+      <c r="F30" s="23" t="n">
+        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$34,$B30,Seguimiento!$I$7:$I$34,"WiFi y cable")</f>
         <v>2</v>
       </c>
-      <c r="F30" s="23" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$33,$B30,Seguimiento!$I$7:$I$33,"Acceso total (WiFi + Cable)")</f>
-        <v>1</v>
-      </c>
       <c r="G30" s="23" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$33,$B30,Seguimiento!$I$7:$I$33,"Solo WiFi")+COUNTIFS(Seguimiento!$C$7:$C$33,$B30,Seguimiento!$I$7:$I$33,"Solo cable Ethernet")</f>
+        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$34,$B30,Seguimiento!$I$7:$I$34,"Solo WiFi")+COUNTIFS(Seguimiento!$C$7:$C$34,$B30,Seguimiento!$I$7:$I$34,"Solo cable")</f>
         <v>0</v>
       </c>
       <c r="H30" s="23" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$33,$B30,Seguimiento!$I$7:$I$33,"Sin acceso")</f>
+        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$34,$B30,Seguimiento!$I$7:$I$34,"Sin acceso")</f>
+        <v>5</v>
+      </c>
+      <c r="I30" s="23" t="n">
+        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$34,$B30,Seguimiento!$I$7:$I$34,"Pendiente")</f>
         <v>0</v>
-      </c>
-      <c r="I30" s="23" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$33,$B30,Seguimiento!$I$7:$I$33,"Pendiente")</f>
-        <v>1</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B31" s="24" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="C31" s="24"/>
       <c r="D31" s="24"/>
       <c r="E31" s="25" t="n">
-        <f aca="false">COUNTIF(Seguimiento!$C$7:$C$33,$B31)</f>
-        <v>3</v>
+        <f aca="false">COUNTIF(Seguimiento!$C$7:$C$34,$B31)</f>
+        <v>2</v>
       </c>
       <c r="F31" s="26" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$33,$B31,Seguimiento!$I$7:$I$33,"Acceso total (WiFi + Cable)")</f>
-        <v>3</v>
+        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$34,$B31,Seguimiento!$I$7:$I$34,"WiFi y cable")</f>
+        <v>1</v>
       </c>
       <c r="G31" s="26" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$33,$B31,Seguimiento!$I$7:$I$33,"Solo WiFi")+COUNTIFS(Seguimiento!$C$7:$C$33,$B31,Seguimiento!$I$7:$I$33,"Solo cable Ethernet")</f>
+        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$34,$B31,Seguimiento!$I$7:$I$34,"Solo WiFi")+COUNTIFS(Seguimiento!$C$7:$C$34,$B31,Seguimiento!$I$7:$I$34,"Solo cable")</f>
         <v>0</v>
       </c>
       <c r="H31" s="26" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$33,$B31,Seguimiento!$I$7:$I$33,"Sin acceso")</f>
+        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$34,$B31,Seguimiento!$I$7:$I$34,"Sin acceso")</f>
         <v>0</v>
       </c>
       <c r="I31" s="26" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$33,$B31,Seguimiento!$I$7:$I$33,"Pendiente")</f>
-        <v>0</v>
+        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$34,$B31,Seguimiento!$I$7:$I$34,"Pendiente")</f>
+        <v>1</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="21" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="C32" s="21"/>
       <c r="D32" s="21"/>
       <c r="E32" s="22" t="n">
-        <f aca="false">COUNTIF(Seguimiento!$C$7:$C$33,$B32)</f>
+        <f aca="false">COUNTIF(Seguimiento!$C$7:$C$34,$B32)</f>
+        <v>3</v>
+      </c>
+      <c r="F32" s="23" t="n">
+        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$34,$B32,Seguimiento!$I$7:$I$34,"WiFi y cable")</f>
+        <v>3</v>
+      </c>
+      <c r="G32" s="23" t="n">
+        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$34,$B32,Seguimiento!$I$7:$I$34,"Solo WiFi")+COUNTIFS(Seguimiento!$C$7:$C$34,$B32,Seguimiento!$I$7:$I$34,"Solo cable")</f>
+        <v>0</v>
+      </c>
+      <c r="H32" s="23" t="n">
+        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$34,$B32,Seguimiento!$I$7:$I$34,"Sin acceso")</f>
+        <v>0</v>
+      </c>
+      <c r="I32" s="23" t="n">
+        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$34,$B32,Seguimiento!$I$7:$I$34,"Pendiente")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B33" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="C33" s="24"/>
+      <c r="D33" s="24"/>
+      <c r="E33" s="25" t="n">
+        <f aca="false">COUNTIF(Seguimiento!$C$7:$C$34,$B33)</f>
         <v>1</v>
       </c>
-      <c r="F32" s="23" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$33,$B32,Seguimiento!$I$7:$I$33,"Acceso total (WiFi + Cable)")</f>
+      <c r="F33" s="26" t="n">
+        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$34,$B33,Seguimiento!$I$7:$I$34,"WiFi y cable")</f>
         <v>0</v>
       </c>
-      <c r="G32" s="23" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$33,$B32,Seguimiento!$I$7:$I$33,"Solo WiFi")+COUNTIFS(Seguimiento!$C$7:$C$33,$B32,Seguimiento!$I$7:$I$33,"Solo cable Ethernet")</f>
+      <c r="G33" s="26" t="n">
+        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$34,$B33,Seguimiento!$I$7:$I$34,"Solo WiFi")+COUNTIFS(Seguimiento!$C$7:$C$34,$B33,Seguimiento!$I$7:$I$34,"Solo cable")</f>
         <v>0</v>
       </c>
-      <c r="H32" s="23" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$33,$B32,Seguimiento!$I$7:$I$33,"Sin acceso")</f>
+      <c r="H33" s="26" t="n">
+        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$34,$B33,Seguimiento!$I$7:$I$34,"Sin acceso")</f>
         <v>0</v>
       </c>
-      <c r="I32" s="23" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$33,$B32,Seguimiento!$I$7:$I$33,"Pendiente")</f>
+      <c r="I33" s="26" t="n">
+        <f aca="false">COUNTIFS(Seguimiento!$C$7:$C$34,$B33,Seguimiento!$I$7:$I$34,"Pendiente")</f>
         <v>1</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B33" s="18" t="s">
-        <v>20</v>
-      </c>
-      <c r="C33" s="18"/>
-      <c r="D33" s="18"/>
-      <c r="E33" s="19" t="n">
-        <f aca="false">SUM(E26:E32)</f>
+    <row r="34" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B34" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="F33" s="19" t="n">
-        <f aca="false">SUM(F26:F32)</f>
-        <v>6</v>
-      </c>
-      <c r="G33" s="19" t="n">
-        <f aca="false">SUM(G26:G32)</f>
+      <c r="C34" s="18"/>
+      <c r="D34" s="18"/>
+      <c r="E34" s="19" t="n">
+        <f aca="false">SUM(E26:E33)</f>
+        <v>18</v>
+      </c>
+      <c r="F34" s="19" t="n">
+        <f aca="false">SUM(F26:F33)</f>
+        <v>7</v>
+      </c>
+      <c r="G34" s="19" t="n">
+        <f aca="false">SUM(G26:G33)</f>
         <v>1</v>
       </c>
-      <c r="H33" s="19" t="n">
-        <f aca="false">SUM(H26:H32)</f>
+      <c r="H34" s="19" t="n">
+        <f aca="false">SUM(H26:H33)</f>
         <v>7</v>
       </c>
-      <c r="I33" s="19" t="n">
-        <f aca="false">SUM(I26:I32)</f>
+      <c r="I34" s="19" t="n">
+        <f aca="false">SUM(I26:I33)</f>
         <v>3</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B34" s="27" t="str">
-        <f aca="false">IF($E$33=COUNTA(Seguimiento!$B$7:$B$33),"Todas las áreas cuadran con la hoja Seguimiento.","Atención: hay sistemas cuya Área funcional no coincide con ninguna fila de esta tabla. Añada el área que falte para que el total vuelva a cuadrar.")</f>
-        <v>Todas las áreas cuadran con la hoja Seguimiento.</v>
-      </c>
-      <c r="C34" s="27"/>
-      <c r="D34" s="27"/>
-      <c r="E34" s="27"/>
-      <c r="F34" s="27"/>
-      <c r="G34" s="27"/>
-      <c r="H34" s="27"/>
-      <c r="I34" s="27"/>
+    <row r="35" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B35" s="27" t="str">
+        <f aca="false">IF($E$34=COUNTA(Seguimiento!$B$7:$B$34),"Cuadra con la hoja Seguimiento.","Ojo: hay sistemas con un área que no aparece en esta tabla. Añádela para que cuadre.")</f>
+        <v>Cuadra con la hoja Seguimiento.</v>
+      </c>
+      <c r="C35" s="27"/>
+      <c r="D35" s="27"/>
+      <c r="E35" s="27"/>
+      <c r="F35" s="27"/>
+      <c r="G35" s="27"/>
+      <c r="H35" s="27"/>
+      <c r="I35" s="27"/>
     </row>
     <row r="38" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="9" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C38" s="9"/>
       <c r="D38" s="9"/>
@@ -3578,17 +3641,17 @@
       <c r="P38" s="9"/>
       <c r="Q38" s="9"/>
     </row>
-    <row r="39" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B39" s="10" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C39" s="10"/>
       <c r="D39" s="10"/>
       <c r="E39" s="11" t="s">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="F39" s="10" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="G39" s="10"/>
       <c r="H39" s="10"/>
@@ -3596,17 +3659,17 @@
     </row>
     <row r="40" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B40" s="21" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C40" s="21"/>
       <c r="D40" s="21"/>
       <c r="E40" s="22" t="n">
-        <f aca="false">COUNTIF(Seguimiento!$M$7:$M$33,$B40)</f>
-        <v>6</v>
+        <f aca="false">COUNTIF(Seguimiento!$M$7:$M$34,$B40)</f>
+        <v>7</v>
       </c>
       <c r="F40" s="28" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$M$7:$M$33,$B40,Seguimiento!$J$7:$J$33,"Crítica")+COUNTIFS(Seguimiento!$M$7:$M$33,$B40,Seguimiento!$J$7:$J$33,"Alta")</f>
-        <v>3</v>
+        <f aca="false">COUNTIFS(Seguimiento!$M$7:$M$34,$B40,Seguimiento!$J$7:$J$34,"Crítica")+COUNTIFS(Seguimiento!$M$7:$M$34,$B40,Seguimiento!$J$7:$J$34,"Alta")</f>
+        <v>4</v>
       </c>
       <c r="G40" s="28"/>
       <c r="H40" s="28"/>
@@ -3614,16 +3677,16 @@
     </row>
     <row r="41" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B41" s="24" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C41" s="24"/>
       <c r="D41" s="24"/>
       <c r="E41" s="25" t="n">
-        <f aca="false">COUNTIF(Seguimiento!$M$7:$M$33,$B41)</f>
+        <f aca="false">COUNTIF(Seguimiento!$M$7:$M$34,$B41)</f>
         <v>1</v>
       </c>
       <c r="F41" s="29" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$M$7:$M$33,$B41,Seguimiento!$J$7:$J$33,"Crítica")+COUNTIFS(Seguimiento!$M$7:$M$33,$B41,Seguimiento!$J$7:$J$33,"Alta")</f>
+        <f aca="false">COUNTIFS(Seguimiento!$M$7:$M$34,$B41,Seguimiento!$J$7:$J$34,"Crítica")+COUNTIFS(Seguimiento!$M$7:$M$34,$B41,Seguimiento!$J$7:$J$34,"Alta")</f>
         <v>1</v>
       </c>
       <c r="G41" s="29"/>
@@ -3632,16 +3695,16 @@
     </row>
     <row r="42" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B42" s="21" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C42" s="21"/>
       <c r="D42" s="21"/>
       <c r="E42" s="22" t="n">
-        <f aca="false">COUNTIF(Seguimiento!$M$7:$M$33,$B42)</f>
+        <f aca="false">COUNTIF(Seguimiento!$M$7:$M$34,$B42)</f>
         <v>2</v>
       </c>
       <c r="F42" s="28" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$M$7:$M$33,$B42,Seguimiento!$J$7:$J$33,"Crítica")+COUNTIFS(Seguimiento!$M$7:$M$33,$B42,Seguimiento!$J$7:$J$33,"Alta")</f>
+        <f aca="false">COUNTIFS(Seguimiento!$M$7:$M$34,$B42,Seguimiento!$J$7:$J$34,"Crítica")+COUNTIFS(Seguimiento!$M$7:$M$34,$B42,Seguimiento!$J$7:$J$34,"Alta")</f>
         <v>2</v>
       </c>
       <c r="G42" s="28"/>
@@ -3650,16 +3713,16 @@
     </row>
     <row r="43" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B43" s="24" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C43" s="24"/>
       <c r="D43" s="24"/>
       <c r="E43" s="25" t="n">
-        <f aca="false">COUNTIF(Seguimiento!$M$7:$M$33,$B43)</f>
+        <f aca="false">COUNTIF(Seguimiento!$M$7:$M$34,$B43)</f>
         <v>7</v>
       </c>
       <c r="F43" s="29" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$M$7:$M$33,$B43,Seguimiento!$J$7:$J$33,"Crítica")+COUNTIFS(Seguimiento!$M$7:$M$33,$B43,Seguimiento!$J$7:$J$33,"Alta")</f>
+        <f aca="false">COUNTIFS(Seguimiento!$M$7:$M$34,$B43,Seguimiento!$J$7:$J$34,"Crítica")+COUNTIFS(Seguimiento!$M$7:$M$34,$B43,Seguimiento!$J$7:$J$34,"Alta")</f>
         <v>5</v>
       </c>
       <c r="G43" s="29"/>
@@ -3668,16 +3731,16 @@
     </row>
     <row r="44" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B44" s="21" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="C44" s="21"/>
       <c r="D44" s="21"/>
       <c r="E44" s="22" t="n">
-        <f aca="false">COUNTIF(Seguimiento!$M$7:$M$33,$B44)</f>
+        <f aca="false">COUNTIF(Seguimiento!$M$7:$M$34,$B44)</f>
         <v>1</v>
       </c>
       <c r="F44" s="28" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$M$7:$M$33,$B44,Seguimiento!$J$7:$J$33,"Crítica")+COUNTIFS(Seguimiento!$M$7:$M$33,$B44,Seguimiento!$J$7:$J$33,"Alta")</f>
+        <f aca="false">COUNTIFS(Seguimiento!$M$7:$M$34,$B44,Seguimiento!$J$7:$J$34,"Crítica")+COUNTIFS(Seguimiento!$M$7:$M$34,$B44,Seguimiento!$J$7:$J$34,"Alta")</f>
         <v>1</v>
       </c>
       <c r="G44" s="28"/>
@@ -3686,16 +3749,16 @@
     </row>
     <row r="45" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B45" s="24" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C45" s="24"/>
       <c r="D45" s="24"/>
       <c r="E45" s="25" t="n">
-        <f aca="false">COUNTIF(Seguimiento!$M$7:$M$33,$B45)</f>
+        <f aca="false">COUNTIF(Seguimiento!$M$7:$M$34,$B45)</f>
         <v>0</v>
       </c>
       <c r="F45" s="29" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$M$7:$M$33,$B45,Seguimiento!$J$7:$J$33,"Crítica")+COUNTIFS(Seguimiento!$M$7:$M$33,$B45,Seguimiento!$J$7:$J$33,"Alta")</f>
+        <f aca="false">COUNTIFS(Seguimiento!$M$7:$M$34,$B45,Seguimiento!$J$7:$J$34,"Crítica")+COUNTIFS(Seguimiento!$M$7:$M$34,$B45,Seguimiento!$J$7:$J$34,"Alta")</f>
         <v>0</v>
       </c>
       <c r="G45" s="29"/>
@@ -3704,16 +3767,16 @@
     </row>
     <row r="46" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B46" s="21" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C46" s="21"/>
       <c r="D46" s="21"/>
       <c r="E46" s="22" t="n">
-        <f aca="false">COUNTIF(Seguimiento!$M$7:$M$33,$B46)</f>
+        <f aca="false">COUNTIF(Seguimiento!$M$7:$M$34,$B46)</f>
         <v>0</v>
       </c>
       <c r="F46" s="28" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$M$7:$M$33,$B46,Seguimiento!$J$7:$J$33,"Crítica")+COUNTIFS(Seguimiento!$M$7:$M$33,$B46,Seguimiento!$J$7:$J$33,"Alta")</f>
+        <f aca="false">COUNTIFS(Seguimiento!$M$7:$M$34,$B46,Seguimiento!$J$7:$J$34,"Crítica")+COUNTIFS(Seguimiento!$M$7:$M$34,$B46,Seguimiento!$J$7:$J$34,"Alta")</f>
         <v>0</v>
       </c>
       <c r="G46" s="28"/>
@@ -3722,16 +3785,16 @@
     </row>
     <row r="47" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B47" s="24" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C47" s="24"/>
       <c r="D47" s="24"/>
       <c r="E47" s="25" t="n">
-        <f aca="false">COUNTIF(Seguimiento!$M$7:$M$33,$B47)</f>
+        <f aca="false">COUNTIF(Seguimiento!$M$7:$M$34,$B47)</f>
         <v>0</v>
       </c>
       <c r="F47" s="29" t="n">
-        <f aca="false">COUNTIFS(Seguimiento!$M$7:$M$33,$B47,Seguimiento!$J$7:$J$33,"Crítica")+COUNTIFS(Seguimiento!$M$7:$M$33,$B47,Seguimiento!$J$7:$J$33,"Alta")</f>
+        <f aca="false">COUNTIFS(Seguimiento!$M$7:$M$34,$B47,Seguimiento!$J$7:$J$34,"Crítica")+COUNTIFS(Seguimiento!$M$7:$M$34,$B47,Seguimiento!$J$7:$J$34,"Alta")</f>
         <v>0</v>
       </c>
       <c r="G47" s="29"/>
@@ -3740,25 +3803,25 @@
     </row>
     <row r="48" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B48" s="18" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C48" s="18"/>
       <c r="D48" s="18"/>
       <c r="E48" s="19" t="n">
         <f aca="false">SUM(E40:E47)</f>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F48" s="19" t="n">
         <f aca="false">SUM(F40:F47)</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G48" s="19"/>
       <c r="H48" s="19"/>
       <c r="I48" s="19"/>
     </row>
-    <row r="50" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B50" s="30" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C50" s="30"/>
       <c r="D50" s="30"/>
@@ -3776,9 +3839,9 @@
       <c r="P50" s="30"/>
       <c r="Q50" s="30"/>
     </row>
-    <row r="51" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B51" s="30" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C51" s="30"/>
       <c r="D51" s="30"/>
@@ -3796,9 +3859,9 @@
       <c r="P51" s="30"/>
       <c r="Q51" s="30"/>
     </row>
-    <row r="52" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B52" s="30" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C52" s="30"/>
       <c r="D52" s="30"/>
@@ -3817,7 +3880,7 @@
       <c r="Q52" s="30"/>
     </row>
   </sheetData>
-  <mergeCells count="62">
+  <mergeCells count="63">
     <mergeCell ref="A1:Q1"/>
     <mergeCell ref="A2:Q2"/>
     <mergeCell ref="B4:D4"/>
@@ -3855,7 +3918,8 @@
     <mergeCell ref="B31:D31"/>
     <mergeCell ref="B32:D32"/>
     <mergeCell ref="B33:D33"/>
-    <mergeCell ref="B34:I34"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="B35:I35"/>
     <mergeCell ref="B38:Q38"/>
     <mergeCell ref="B39:D39"/>
     <mergeCell ref="F39:I39"/>
@@ -3898,28 +3962,27 @@
     <tabColor rgb="FFD99B2B"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:N44"/>
+  <dimension ref="A1:N45"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="50"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3937,7 +4000,7 @@
     </row>
     <row r="2" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3953,9 +4016,9 @@
       <c r="M2" s="2"/>
       <c r="N2" s="2"/>
     </row>
-    <row r="3" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="31" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B3" s="31"/>
       <c r="C3" s="31"/>
@@ -3973,797 +4036,790 @@
     </row>
     <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="32" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B4" s="32"/>
       <c r="C4" s="33" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="D4" s="33"/>
       <c r="E4" s="34" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F4" s="34"/>
       <c r="G4" s="35" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="H4" s="35"/>
       <c r="I4" s="36" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="J4" s="36"/>
       <c r="K4" s="37" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="L4" s="37"/>
       <c r="M4" s="37"/>
       <c r="N4" s="37"/>
     </row>
     <row r="5" customFormat="false" ht="6.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="6" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="B6" s="38" t="s">
+        <v>52</v>
+      </c>
+      <c r="C6" s="38" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="38" t="s">
+        <v>53</v>
+      </c>
+      <c r="E6" s="38" t="s">
+        <v>54</v>
+      </c>
+      <c r="F6" s="38" t="s">
         <v>55</v>
       </c>
-      <c r="B6" s="38" t="s">
+      <c r="G6" s="38" t="s">
         <v>56</v>
       </c>
-      <c r="C6" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="D6" s="38" t="s">
+      <c r="H6" s="38" t="s">
         <v>57</v>
-      </c>
-      <c r="E6" s="38" t="s">
-        <v>58</v>
-      </c>
-      <c r="F6" s="38" t="s">
-        <v>59</v>
-      </c>
-      <c r="G6" s="38" t="s">
-        <v>60</v>
-      </c>
-      <c r="H6" s="38" t="s">
-        <v>61</v>
       </c>
       <c r="I6" s="38" t="s">
         <v>11</v>
       </c>
       <c r="J6" s="38" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="K6" s="38" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="L6" s="38" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="M6" s="38" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="N6" s="38" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="39" t="n">
         <v>1</v>
       </c>
       <c r="B7" s="40" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>25</v>
-      </c>
-      <c r="D7" s="41" t="s">
-        <v>67</v>
-      </c>
-      <c r="E7" s="42" t="s">
-        <v>68</v>
-      </c>
-      <c r="F7" s="43" t="s">
-        <v>69</v>
+        <v>20</v>
+      </c>
+      <c r="D7" s="41"/>
+      <c r="E7" s="41"/>
+      <c r="F7" s="42" t="s">
+        <v>63</v>
       </c>
       <c r="G7" s="43" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="H7" s="43" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="I7" s="44" t="str">
-        <f aca="false">IF($B7="","",IF($F7="No aplica","No aplica",IF(AND($G7="OK",$H7="OK"),"Acceso total (WiFi + Cable)",IF(AND($G7="OK",$H7&lt;&gt;"OK"),"Solo WiFi",IF(AND($H7="OK",$G7&lt;&gt;"OK"),"Solo cable Ethernet",IF(AND($G7="KO",$H7="KO"),"Sin acceso","Pendiente"))))))</f>
-        <v>Pendiente</v>
+        <f aca="false">IF($B7="","",IF($F7="No aplica","No aplica",IF(AND($G7="OK",$H7="OK"),"WiFi y cable",IF(AND($G7="OK",$H7&lt;&gt;"OK"),"Solo WiFi",IF(AND($H7="OK",$G7&lt;&gt;"OK"),"Solo cable",IF(AND($G7="KO",$H7="KO"),"Sin acceso","Pendiente"))))))</f>
+        <v>WiFi y cable</v>
       </c>
       <c r="J7" s="43" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="K7" s="45"/>
       <c r="L7" s="46"/>
-      <c r="M7" s="43" t="s">
-        <v>36</v>
+      <c r="M7" s="42" t="s">
+        <v>31</v>
       </c>
       <c r="N7" s="47" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="48" t="n">
         <v>2</v>
       </c>
       <c r="B8" s="49" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C8" s="50" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="D8" s="50" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="E8" s="51" t="s">
-        <v>75</v>
-      </c>
-      <c r="F8" s="43" t="s">
-        <v>76</v>
+        <v>69</v>
+      </c>
+      <c r="F8" s="42" t="s">
+        <v>70</v>
       </c>
       <c r="G8" s="43" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="H8" s="43" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="I8" s="52" t="str">
-        <f aca="false">IF($B8="","",IF($F8="No aplica","No aplica",IF(AND($G8="OK",$H8="OK"),"Acceso total (WiFi + Cable)",IF(AND($G8="OK",$H8&lt;&gt;"OK"),"Solo WiFi",IF(AND($H8="OK",$G8&lt;&gt;"OK"),"Solo cable Ethernet",IF(AND($G8="KO",$H8="KO"),"Sin acceso","Pendiente"))))))</f>
-        <v>Solo WiFi</v>
+        <f aca="false">IF($B8="","",IF($F8="No aplica","No aplica",IF(AND($G8="OK",$H8="OK"),"WiFi y cable",IF(AND($G8="OK",$H8&lt;&gt;"OK"),"Solo WiFi",IF(AND($H8="OK",$G8&lt;&gt;"OK"),"Solo cable",IF(AND($G8="KO",$H8="KO"),"Sin acceso","Pendiente"))))))</f>
+        <v>Pendiente</v>
       </c>
       <c r="J8" s="43" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="K8" s="45"/>
       <c r="L8" s="46"/>
-      <c r="M8" s="43" t="s">
-        <v>39</v>
+      <c r="M8" s="42" t="s">
+        <v>32</v>
       </c>
       <c r="N8" s="47" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="39" t="n">
         <v>3</v>
       </c>
       <c r="B9" s="40" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="C9" s="41" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="D9" s="41" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="E9" s="53" t="s">
-        <v>82</v>
-      </c>
-      <c r="F9" s="43" t="s">
+        <v>75</v>
+      </c>
+      <c r="F9" s="42" t="s">
+        <v>63</v>
+      </c>
+      <c r="G9" s="43" t="s">
+        <v>64</v>
+      </c>
+      <c r="H9" s="43" t="s">
         <v>76</v>
       </c>
-      <c r="G9" s="43" t="s">
-        <v>78</v>
-      </c>
-      <c r="H9" s="43" t="s">
-        <v>78</v>
-      </c>
       <c r="I9" s="44" t="str">
-        <f aca="false">IF($B9="","",IF($F9="No aplica","No aplica",IF(AND($G9="OK",$H9="OK"),"Acceso total (WiFi + Cable)",IF(AND($G9="OK",$H9&lt;&gt;"OK"),"Solo WiFi",IF(AND($H9="OK",$G9&lt;&gt;"OK"),"Solo cable Ethernet",IF(AND($G9="KO",$H9="KO"),"Sin acceso","Pendiente"))))))</f>
-        <v>Sin acceso</v>
+        <f aca="false">IF($B9="","",IF($F9="No aplica","No aplica",IF(AND($G9="OK",$H9="OK"),"WiFi y cable",IF(AND($G9="OK",$H9&lt;&gt;"OK"),"Solo WiFi",IF(AND($H9="OK",$G9&lt;&gt;"OK"),"Solo cable",IF(AND($G9="KO",$H9="KO"),"Sin acceso","Pendiente"))))))</f>
+        <v>Solo WiFi</v>
       </c>
       <c r="J9" s="43" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="K9" s="45"/>
       <c r="L9" s="46"/>
-      <c r="M9" s="43" t="s">
-        <v>38</v>
+      <c r="M9" s="42" t="s">
+        <v>35</v>
       </c>
       <c r="N9" s="47" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="48" t="n">
         <v>4</v>
       </c>
       <c r="B10" s="49" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="C10" s="50" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="D10" s="50" t="s">
-        <v>86</v>
-      </c>
-      <c r="E10" s="51" t="s">
-        <v>87</v>
-      </c>
-      <c r="F10" s="43" t="s">
+        <v>79</v>
+      </c>
+      <c r="E10" s="54" t="s">
+        <v>80</v>
+      </c>
+      <c r="F10" s="42" t="s">
+        <v>63</v>
+      </c>
+      <c r="G10" s="43" t="s">
         <v>76</v>
       </c>
-      <c r="G10" s="43" t="s">
-        <v>77</v>
-      </c>
       <c r="H10" s="43" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="I10" s="52" t="str">
-        <f aca="false">IF($B10="","",IF($F10="No aplica","No aplica",IF(AND($G10="OK",$H10="OK"),"Acceso total (WiFi + Cable)",IF(AND($G10="OK",$H10&lt;&gt;"OK"),"Solo WiFi",IF(AND($H10="OK",$G10&lt;&gt;"OK"),"Solo cable Ethernet",IF(AND($G10="KO",$H10="KO"),"Sin acceso","Pendiente"))))))</f>
-        <v>Acceso total (WiFi + Cable)</v>
+        <f aca="false">IF($B10="","",IF($F10="No aplica","No aplica",IF(AND($G10="OK",$H10="OK"),"WiFi y cable",IF(AND($G10="OK",$H10&lt;&gt;"OK"),"Solo WiFi",IF(AND($H10="OK",$G10&lt;&gt;"OK"),"Solo cable",IF(AND($G10="KO",$H10="KO"),"Sin acceso","Pendiente"))))))</f>
+        <v>Sin acceso</v>
       </c>
       <c r="J10" s="43" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="K10" s="45"/>
       <c r="L10" s="46"/>
-      <c r="M10" s="43" t="s">
-        <v>35</v>
+      <c r="M10" s="42" t="s">
+        <v>34</v>
       </c>
       <c r="N10" s="47" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="39" t="n">
         <v>5</v>
       </c>
       <c r="B11" s="40" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="C11" s="41" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="D11" s="41" t="s">
+        <v>84</v>
+      </c>
+      <c r="E11" s="53" t="s">
+        <v>85</v>
+      </c>
+      <c r="F11" s="42" t="s">
+        <v>63</v>
+      </c>
+      <c r="G11" s="43" t="s">
+        <v>64</v>
+      </c>
+      <c r="H11" s="43" t="s">
+        <v>64</v>
+      </c>
+      <c r="I11" s="44" t="str">
+        <f aca="false">IF($B11="","",IF($F11="No aplica","No aplica",IF(AND($G11="OK",$H11="OK"),"WiFi y cable",IF(AND($G11="OK",$H11&lt;&gt;"OK"),"Solo WiFi",IF(AND($H11="OK",$G11&lt;&gt;"OK"),"Solo cable",IF(AND($G11="KO",$H11="KO"),"Sin acceso","Pendiente"))))))</f>
+        <v>WiFi y cable</v>
+      </c>
+      <c r="J11" s="43" t="s">
         <v>86</v>
-      </c>
-      <c r="E11" s="53" t="s">
-        <v>91</v>
-      </c>
-      <c r="F11" s="43" t="s">
-        <v>76</v>
-      </c>
-      <c r="G11" s="43" t="s">
-        <v>77</v>
-      </c>
-      <c r="H11" s="43" t="s">
-        <v>77</v>
-      </c>
-      <c r="I11" s="44" t="str">
-        <f aca="false">IF($B11="","",IF($F11="No aplica","No aplica",IF(AND($G11="OK",$H11="OK"),"Acceso total (WiFi + Cable)",IF(AND($G11="OK",$H11&lt;&gt;"OK"),"Solo WiFi",IF(AND($H11="OK",$G11&lt;&gt;"OK"),"Solo cable Ethernet",IF(AND($G11="KO",$H11="KO"),"Sin acceso","Pendiente"))))))</f>
-        <v>Acceso total (WiFi + Cable)</v>
-      </c>
-      <c r="J11" s="43" t="s">
-        <v>88</v>
       </c>
       <c r="K11" s="45"/>
       <c r="L11" s="46"/>
-      <c r="M11" s="43" t="s">
-        <v>35</v>
-      </c>
-      <c r="N11" s="47" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="M11" s="42" t="s">
+        <v>31</v>
+      </c>
+      <c r="N11" s="47"/>
+    </row>
+    <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="48" t="n">
         <v>6</v>
       </c>
       <c r="B12" s="49" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="C12" s="50" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D12" s="50" t="s">
-        <v>93</v>
-      </c>
-      <c r="E12" s="51" t="s">
-        <v>94</v>
-      </c>
-      <c r="F12" s="43" t="s">
-        <v>76</v>
+        <v>84</v>
+      </c>
+      <c r="E12" s="54" t="s">
+        <v>88</v>
+      </c>
+      <c r="F12" s="42" t="s">
+        <v>63</v>
       </c>
       <c r="G12" s="43" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="H12" s="43" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="I12" s="52" t="str">
-        <f aca="false">IF($B12="","",IF($F12="No aplica","No aplica",IF(AND($G12="OK",$H12="OK"),"Acceso total (WiFi + Cable)",IF(AND($G12="OK",$H12&lt;&gt;"OK"),"Solo WiFi",IF(AND($H12="OK",$G12&lt;&gt;"OK"),"Solo cable Ethernet",IF(AND($G12="KO",$H12="KO"),"Sin acceso","Pendiente"))))))</f>
-        <v>Acceso total (WiFi + Cable)</v>
+        <f aca="false">IF($B12="","",IF($F12="No aplica","No aplica",IF(AND($G12="OK",$H12="OK"),"WiFi y cable",IF(AND($G12="OK",$H12&lt;&gt;"OK"),"Solo WiFi",IF(AND($H12="OK",$G12&lt;&gt;"OK"),"Solo cable",IF(AND($G12="KO",$H12="KO"),"Sin acceso","Pendiente"))))))</f>
+        <v>WiFi y cable</v>
       </c>
       <c r="J12" s="43" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="K12" s="45"/>
       <c r="L12" s="46"/>
-      <c r="M12" s="43" t="s">
-        <v>35</v>
-      </c>
-      <c r="N12" s="47" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="M12" s="42" t="s">
+        <v>31</v>
+      </c>
+      <c r="N12" s="47"/>
+    </row>
+    <row r="13" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="39" t="n">
         <v>7</v>
       </c>
       <c r="B13" s="40" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="C13" s="41" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="D13" s="41" t="s">
-        <v>96</v>
-      </c>
-      <c r="E13" s="42" t="s">
-        <v>97</v>
-      </c>
-      <c r="F13" s="43" t="s">
-        <v>98</v>
+        <v>90</v>
+      </c>
+      <c r="E13" s="53" t="s">
+        <v>91</v>
+      </c>
+      <c r="F13" s="42" t="s">
+        <v>63</v>
       </c>
       <c r="G13" s="43" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="H13" s="43" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="I13" s="44" t="str">
-        <f aca="false">IF($B13="","",IF($F13="No aplica","No aplica",IF(AND($G13="OK",$H13="OK"),"Acceso total (WiFi + Cable)",IF(AND($G13="OK",$H13&lt;&gt;"OK"),"Solo WiFi",IF(AND($H13="OK",$G13&lt;&gt;"OK"),"Solo cable Ethernet",IF(AND($G13="KO",$H13="KO"),"Sin acceso","Pendiente"))))))</f>
-        <v>Pendiente</v>
+        <f aca="false">IF($B13="","",IF($F13="No aplica","No aplica",IF(AND($G13="OK",$H13="OK"),"WiFi y cable",IF(AND($G13="OK",$H13&lt;&gt;"OK"),"Solo WiFi",IF(AND($H13="OK",$G13&lt;&gt;"OK"),"Solo cable",IF(AND($G13="KO",$H13="KO"),"Sin acceso","Pendiente"))))))</f>
+        <v>WiFi y cable</v>
       </c>
       <c r="J13" s="43" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="K13" s="45"/>
       <c r="L13" s="46"/>
-      <c r="M13" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="N13" s="47" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="M13" s="42" t="s">
+        <v>31</v>
+      </c>
+      <c r="N13" s="47"/>
+    </row>
+    <row r="14" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="48" t="n">
         <v>8</v>
       </c>
       <c r="B14" s="49" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="C14" s="50" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D14" s="50" t="s">
         <v>93</v>
       </c>
-      <c r="E14" s="54" t="s">
-        <v>101</v>
-      </c>
-      <c r="F14" s="43" t="s">
-        <v>98</v>
+      <c r="E14" s="51" t="s">
+        <v>94</v>
+      </c>
+      <c r="F14" s="42" t="s">
+        <v>95</v>
       </c>
       <c r="G14" s="43" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H14" s="43" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="I14" s="52" t="str">
-        <f aca="false">IF($B14="","",IF($F14="No aplica","No aplica",IF(AND($G14="OK",$H14="OK"),"Acceso total (WiFi + Cable)",IF(AND($G14="OK",$H14&lt;&gt;"OK"),"Solo WiFi",IF(AND($H14="OK",$G14&lt;&gt;"OK"),"Solo cable Ethernet",IF(AND($G14="KO",$H14="KO"),"Sin acceso","Pendiente"))))))</f>
+        <f aca="false">IF($B14="","",IF($F14="No aplica","No aplica",IF(AND($G14="OK",$H14="OK"),"WiFi y cable",IF(AND($G14="OK",$H14&lt;&gt;"OK"),"Solo WiFi",IF(AND($H14="OK",$G14&lt;&gt;"OK"),"Solo cable",IF(AND($G14="KO",$H14="KO"),"Sin acceso","Pendiente"))))))</f>
         <v>Pendiente</v>
       </c>
       <c r="J14" s="43" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="K14" s="45"/>
       <c r="L14" s="46"/>
-      <c r="M14" s="43" t="s">
-        <v>37</v>
+      <c r="M14" s="42" t="s">
+        <v>33</v>
       </c>
       <c r="N14" s="47" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="39" t="n">
         <v>9</v>
       </c>
       <c r="B15" s="40" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="C15" s="41" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="D15" s="41" t="s">
-        <v>86</v>
-      </c>
-      <c r="E15" s="53" t="s">
-        <v>103</v>
-      </c>
-      <c r="F15" s="43" t="s">
-        <v>76</v>
+        <v>90</v>
+      </c>
+      <c r="E15" s="55" t="s">
+        <v>98</v>
+      </c>
+      <c r="F15" s="42" t="s">
+        <v>95</v>
       </c>
       <c r="G15" s="43" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="H15" s="43" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="I15" s="44" t="str">
-        <f aca="false">IF($B15="","",IF($F15="No aplica","No aplica",IF(AND($G15="OK",$H15="OK"),"Acceso total (WiFi + Cable)",IF(AND($G15="OK",$H15&lt;&gt;"OK"),"Solo WiFi",IF(AND($H15="OK",$G15&lt;&gt;"OK"),"Solo cable Ethernet",IF(AND($G15="KO",$H15="KO"),"Sin acceso","Pendiente"))))))</f>
-        <v>Acceso total (WiFi + Cable)</v>
+        <f aca="false">IF($B15="","",IF($F15="No aplica","No aplica",IF(AND($G15="OK",$H15="OK"),"WiFi y cable",IF(AND($G15="OK",$H15&lt;&gt;"OK"),"Solo WiFi",IF(AND($H15="OK",$G15&lt;&gt;"OK"),"Solo cable",IF(AND($G15="KO",$H15="KO"),"Sin acceso","Pendiente"))))))</f>
+        <v>Pendiente</v>
       </c>
       <c r="J15" s="43" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="K15" s="45"/>
       <c r="L15" s="46"/>
-      <c r="M15" s="43" t="s">
-        <v>35</v>
+      <c r="M15" s="42" t="s">
+        <v>33</v>
       </c>
       <c r="N15" s="47" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="48" t="n">
         <v>10</v>
       </c>
       <c r="B16" s="49" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="C16" s="50" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D16" s="50" t="s">
-        <v>105</v>
-      </c>
-      <c r="E16" s="51" t="s">
-        <v>106</v>
-      </c>
-      <c r="F16" s="43" t="s">
-        <v>76</v>
+        <v>84</v>
+      </c>
+      <c r="E16" s="54" t="s">
+        <v>100</v>
+      </c>
+      <c r="F16" s="42" t="s">
+        <v>63</v>
       </c>
       <c r="G16" s="43" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="H16" s="43" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="I16" s="52" t="str">
-        <f aca="false">IF($B16="","",IF($F16="No aplica","No aplica",IF(AND($G16="OK",$H16="OK"),"Acceso total (WiFi + Cable)",IF(AND($G16="OK",$H16&lt;&gt;"OK"),"Solo WiFi",IF(AND($H16="OK",$G16&lt;&gt;"OK"),"Solo cable Ethernet",IF(AND($G16="KO",$H16="KO"),"Sin acceso","Pendiente"))))))</f>
-        <v>Sin acceso</v>
+        <f aca="false">IF($B16="","",IF($F16="No aplica","No aplica",IF(AND($G16="OK",$H16="OK"),"WiFi y cable",IF(AND($G16="OK",$H16&lt;&gt;"OK"),"Solo WiFi",IF(AND($H16="OK",$G16&lt;&gt;"OK"),"Solo cable",IF(AND($G16="KO",$H16="KO"),"Sin acceso","Pendiente"))))))</f>
+        <v>WiFi y cable</v>
       </c>
       <c r="J16" s="43" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="K16" s="45"/>
       <c r="L16" s="46"/>
-      <c r="M16" s="43" t="s">
-        <v>38</v>
-      </c>
-      <c r="N16" s="47" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="M16" s="42" t="s">
+        <v>31</v>
+      </c>
+      <c r="N16" s="47"/>
+    </row>
+    <row r="17" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="39" t="n">
         <v>11</v>
       </c>
       <c r="B17" s="40" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="C17" s="41" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D17" s="41" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="E17" s="53" t="s">
-        <v>109</v>
-      </c>
-      <c r="F17" s="43" t="s">
+        <v>103</v>
+      </c>
+      <c r="F17" s="42" t="s">
+        <v>63</v>
+      </c>
+      <c r="G17" s="43" t="s">
         <v>76</v>
       </c>
-      <c r="G17" s="43" t="s">
-        <v>77</v>
-      </c>
       <c r="H17" s="43" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="I17" s="44" t="str">
-        <f aca="false">IF($B17="","",IF($F17="No aplica","No aplica",IF(AND($G17="OK",$H17="OK"),"Acceso total (WiFi + Cable)",IF(AND($G17="OK",$H17&lt;&gt;"OK"),"Solo WiFi",IF(AND($H17="OK",$G17&lt;&gt;"OK"),"Solo cable Ethernet",IF(AND($G17="KO",$H17="KO"),"Sin acceso","Pendiente"))))))</f>
-        <v>Acceso total (WiFi + Cable)</v>
+        <f aca="false">IF($B17="","",IF($F17="No aplica","No aplica",IF(AND($G17="OK",$H17="OK"),"WiFi y cable",IF(AND($G17="OK",$H17&lt;&gt;"OK"),"Solo WiFi",IF(AND($H17="OK",$G17&lt;&gt;"OK"),"Solo cable",IF(AND($G17="KO",$H17="KO"),"Sin acceso","Pendiente"))))))</f>
+        <v>Sin acceso</v>
       </c>
       <c r="J17" s="43" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="K17" s="45"/>
       <c r="L17" s="46"/>
-      <c r="M17" s="43" t="s">
-        <v>35</v>
-      </c>
-      <c r="N17" s="47" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="M17" s="42" t="s">
+        <v>34</v>
+      </c>
+      <c r="N17" s="47"/>
+    </row>
+    <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="48" t="n">
         <v>12</v>
       </c>
       <c r="B18" s="49" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="C18" s="50" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D18" s="50" t="s">
-        <v>86</v>
-      </c>
-      <c r="E18" s="51" t="s">
-        <v>112</v>
-      </c>
-      <c r="F18" s="43" t="s">
-        <v>76</v>
+        <v>102</v>
+      </c>
+      <c r="E18" s="54" t="s">
+        <v>105</v>
+      </c>
+      <c r="F18" s="42" t="s">
+        <v>63</v>
       </c>
       <c r="G18" s="43" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="H18" s="43" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="I18" s="52" t="str">
-        <f aca="false">IF($B18="","",IF($F18="No aplica","No aplica",IF(AND($G18="OK",$H18="OK"),"Acceso total (WiFi + Cable)",IF(AND($G18="OK",$H18&lt;&gt;"OK"),"Solo WiFi",IF(AND($H18="OK",$G18&lt;&gt;"OK"),"Solo cable Ethernet",IF(AND($G18="KO",$H18="KO"),"Sin acceso","Pendiente"))))))</f>
-        <v>Acceso total (WiFi + Cable)</v>
+        <f aca="false">IF($B18="","",IF($F18="No aplica","No aplica",IF(AND($G18="OK",$H18="OK"),"WiFi y cable",IF(AND($G18="OK",$H18&lt;&gt;"OK"),"Solo WiFi",IF(AND($H18="OK",$G18&lt;&gt;"OK"),"Solo cable",IF(AND($G18="KO",$H18="KO"),"Sin acceso","Pendiente"))))))</f>
+        <v>WiFi y cable</v>
       </c>
       <c r="J18" s="43" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="K18" s="45"/>
       <c r="L18" s="46"/>
-      <c r="M18" s="43" t="s">
-        <v>35</v>
-      </c>
-      <c r="N18" s="47" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="M18" s="42" t="s">
+        <v>31</v>
+      </c>
+      <c r="N18" s="47"/>
+    </row>
+    <row r="19" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="39" t="n">
         <v>13</v>
       </c>
       <c r="B19" s="40" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="C19" s="41" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D19" s="41" t="s">
-        <v>86</v>
-      </c>
-      <c r="E19" s="42" t="s">
-        <v>114</v>
-      </c>
-      <c r="F19" s="43" t="s">
-        <v>76</v>
+        <v>84</v>
+      </c>
+      <c r="E19" s="53" t="s">
+        <v>107</v>
+      </c>
+      <c r="F19" s="42" t="s">
+        <v>63</v>
       </c>
       <c r="G19" s="43" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="H19" s="43" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="I19" s="44" t="str">
-        <f aca="false">IF($B19="","",IF($F19="No aplica","No aplica",IF(AND($G19="OK",$H19="OK"),"Acceso total (WiFi + Cable)",IF(AND($G19="OK",$H19&lt;&gt;"OK"),"Solo WiFi",IF(AND($H19="OK",$G19&lt;&gt;"OK"),"Solo cable Ethernet",IF(AND($G19="KO",$H19="KO"),"Sin acceso","Pendiente"))))))</f>
-        <v>Sin acceso</v>
+        <f aca="false">IF($B19="","",IF($F19="No aplica","No aplica",IF(AND($G19="OK",$H19="OK"),"WiFi y cable",IF(AND($G19="OK",$H19&lt;&gt;"OK"),"Solo WiFi",IF(AND($H19="OK",$G19&lt;&gt;"OK"),"Solo cable",IF(AND($G19="KO",$H19="KO"),"Sin acceso","Pendiente"))))))</f>
+        <v>WiFi y cable</v>
       </c>
       <c r="J19" s="43" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="K19" s="45"/>
       <c r="L19" s="46"/>
-      <c r="M19" s="43" t="s">
-        <v>38</v>
-      </c>
-      <c r="N19" s="47" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="M19" s="42" t="s">
+        <v>31</v>
+      </c>
+      <c r="N19" s="47"/>
+    </row>
+    <row r="20" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="48" t="n">
         <v>14</v>
       </c>
       <c r="B20" s="49" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="C20" s="50" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D20" s="50" t="s">
-        <v>86</v>
-      </c>
-      <c r="E20" s="51" t="s">
-        <v>117</v>
-      </c>
-      <c r="F20" s="43" t="s">
+        <v>84</v>
+      </c>
+      <c r="E20" s="50"/>
+      <c r="F20" s="42" t="s">
+        <v>63</v>
+      </c>
+      <c r="G20" s="43" t="s">
         <v>76</v>
       </c>
-      <c r="G20" s="43" t="s">
-        <v>78</v>
-      </c>
       <c r="H20" s="43" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="I20" s="52" t="str">
-        <f aca="false">IF($B20="","",IF($F20="No aplica","No aplica",IF(AND($G20="OK",$H20="OK"),"Acceso total (WiFi + Cable)",IF(AND($G20="OK",$H20&lt;&gt;"OK"),"Solo WiFi",IF(AND($H20="OK",$G20&lt;&gt;"OK"),"Solo cable Ethernet",IF(AND($G20="KO",$H20="KO"),"Sin acceso","Pendiente"))))))</f>
+        <f aca="false">IF($B20="","",IF($F20="No aplica","No aplica",IF(AND($G20="OK",$H20="OK"),"WiFi y cable",IF(AND($G20="OK",$H20&lt;&gt;"OK"),"Solo WiFi",IF(AND($H20="OK",$G20&lt;&gt;"OK"),"Solo cable",IF(AND($G20="KO",$H20="KO"),"Sin acceso","Pendiente"))))))</f>
         <v>Sin acceso</v>
       </c>
       <c r="J20" s="43" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="K20" s="45"/>
       <c r="L20" s="46"/>
-      <c r="M20" s="43" t="s">
-        <v>38</v>
+      <c r="M20" s="42" t="s">
+        <v>34</v>
       </c>
       <c r="N20" s="47" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="39" t="n">
         <v>15</v>
       </c>
       <c r="B21" s="40" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="C21" s="41" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D21" s="41" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E21" s="53" t="s">
-        <v>119</v>
-      </c>
-      <c r="F21" s="43" t="s">
+        <v>111</v>
+      </c>
+      <c r="F21" s="42" t="s">
+        <v>63</v>
+      </c>
+      <c r="G21" s="43" t="s">
         <v>76</v>
       </c>
-      <c r="G21" s="43" t="s">
-        <v>78</v>
-      </c>
       <c r="H21" s="43" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="I21" s="44" t="str">
-        <f aca="false">IF($B21="","",IF($F21="No aplica","No aplica",IF(AND($G21="OK",$H21="OK"),"Acceso total (WiFi + Cable)",IF(AND($G21="OK",$H21&lt;&gt;"OK"),"Solo WiFi",IF(AND($H21="OK",$G21&lt;&gt;"OK"),"Solo cable Ethernet",IF(AND($G21="KO",$H21="KO"),"Sin acceso","Pendiente"))))))</f>
+        <f aca="false">IF($B21="","",IF($F21="No aplica","No aplica",IF(AND($G21="OK",$H21="OK"),"WiFi y cable",IF(AND($G21="OK",$H21&lt;&gt;"OK"),"Solo WiFi",IF(AND($H21="OK",$G21&lt;&gt;"OK"),"Solo cable",IF(AND($G21="KO",$H21="KO"),"Sin acceso","Pendiente"))))))</f>
         <v>Sin acceso</v>
       </c>
       <c r="J21" s="43" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="K21" s="45"/>
       <c r="L21" s="46"/>
-      <c r="M21" s="43" t="s">
-        <v>38</v>
-      </c>
-      <c r="N21" s="47" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="M21" s="42" t="s">
+        <v>34</v>
+      </c>
+      <c r="N21" s="47"/>
+    </row>
+    <row r="22" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="48" t="n">
         <v>16</v>
       </c>
       <c r="B22" s="49" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="C22" s="50" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D22" s="50" t="s">
-        <v>121</v>
-      </c>
-      <c r="E22" s="51" t="s">
-        <v>122</v>
-      </c>
-      <c r="F22" s="43" t="s">
+        <v>84</v>
+      </c>
+      <c r="E22" s="54" t="s">
+        <v>113</v>
+      </c>
+      <c r="F22" s="42" t="s">
+        <v>63</v>
+      </c>
+      <c r="G22" s="43" t="s">
         <v>76</v>
       </c>
-      <c r="G22" s="43" t="s">
-        <v>78</v>
-      </c>
       <c r="H22" s="43" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="I22" s="52" t="str">
-        <f aca="false">IF($B22="","",IF($F22="No aplica","No aplica",IF(AND($G22="OK",$H22="OK"),"Acceso total (WiFi + Cable)",IF(AND($G22="OK",$H22&lt;&gt;"OK"),"Solo WiFi",IF(AND($H22="OK",$G22&lt;&gt;"OK"),"Solo cable Ethernet",IF(AND($G22="KO",$H22="KO"),"Sin acceso","Pendiente"))))))</f>
+        <f aca="false">IF($B22="","",IF($F22="No aplica","No aplica",IF(AND($G22="OK",$H22="OK"),"WiFi y cable",IF(AND($G22="OK",$H22&lt;&gt;"OK"),"Solo WiFi",IF(AND($H22="OK",$G22&lt;&gt;"OK"),"Solo cable",IF(AND($G22="KO",$H22="KO"),"Sin acceso","Pendiente"))))))</f>
         <v>Sin acceso</v>
       </c>
       <c r="J22" s="43" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="K22" s="45"/>
       <c r="L22" s="46"/>
-      <c r="M22" s="43" t="s">
-        <v>38</v>
-      </c>
-      <c r="N22" s="47" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="55" t="n">
+      <c r="M22" s="42" t="s">
+        <v>34</v>
+      </c>
+      <c r="N22" s="47"/>
+    </row>
+    <row r="23" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="39" t="n">
         <v>17</v>
       </c>
-      <c r="B23" s="56" t="s">
-        <v>124</v>
-      </c>
-      <c r="C23" s="57" t="s">
+      <c r="B23" s="40" t="s">
+        <v>114</v>
+      </c>
+      <c r="C23" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="D23" s="41" t="s">
+        <v>115</v>
+      </c>
+      <c r="E23" s="53" t="s">
+        <v>116</v>
+      </c>
+      <c r="F23" s="42" t="s">
+        <v>63</v>
+      </c>
+      <c r="G23" s="43" t="s">
+        <v>76</v>
+      </c>
+      <c r="H23" s="43" t="s">
+        <v>76</v>
+      </c>
+      <c r="I23" s="44" t="str">
+        <f aca="false">IF($B23="","",IF($F23="No aplica","No aplica",IF(AND($G23="OK",$H23="OK"),"WiFi y cable",IF(AND($G23="OK",$H23&lt;&gt;"OK"),"Solo WiFi",IF(AND($H23="OK",$G23&lt;&gt;"OK"),"Solo cable",IF(AND($G23="KO",$H23="KO"),"Sin acceso","Pendiente"))))))</f>
+        <v>Sin acceso</v>
+      </c>
+      <c r="J23" s="43" t="s">
+        <v>86</v>
+      </c>
+      <c r="K23" s="45"/>
+      <c r="L23" s="46"/>
+      <c r="M23" s="42" t="s">
+        <v>34</v>
+      </c>
+      <c r="N23" s="47" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="56" t="n">
+        <v>18</v>
+      </c>
+      <c r="B24" s="57" t="s">
+        <v>118</v>
+      </c>
+      <c r="C24" s="58" t="s">
+        <v>23</v>
+      </c>
+      <c r="D24" s="58" t="s">
+        <v>79</v>
+      </c>
+      <c r="E24" s="59" t="s">
         <v>27</v>
       </c>
-      <c r="D23" s="57" t="s">
+      <c r="F24" s="60" t="s">
+        <v>63</v>
+      </c>
+      <c r="G24" s="61" t="s">
+        <v>76</v>
+      </c>
+      <c r="H24" s="61" t="s">
+        <v>76</v>
+      </c>
+      <c r="I24" s="62" t="str">
+        <f aca="false">IF($B24="","",IF($F24="No aplica","No aplica",IF(AND($G24="OK",$H24="OK"),"WiFi y cable",IF(AND($G24="OK",$H24&lt;&gt;"OK"),"Solo WiFi",IF(AND($H24="OK",$G24&lt;&gt;"OK"),"Solo cable",IF(AND($G24="KO",$H24="KO"),"Sin acceso","Pendiente"))))))</f>
+        <v>Sin acceso</v>
+      </c>
+      <c r="J24" s="61" t="s">
         <v>81</v>
       </c>
-      <c r="E23" s="58" t="s">
-        <v>125</v>
-      </c>
-      <c r="F23" s="59" t="s">
-        <v>76</v>
-      </c>
-      <c r="G23" s="59" t="s">
-        <v>78</v>
-      </c>
-      <c r="H23" s="59" t="s">
-        <v>78</v>
-      </c>
-      <c r="I23" s="60" t="str">
-        <f aca="false">IF($B23="","",IF($F23="No aplica","No aplica",IF(AND($G23="OK",$H23="OK"),"Acceso total (WiFi + Cable)",IF(AND($G23="OK",$H23&lt;&gt;"OK"),"Solo WiFi",IF(AND($H23="OK",$G23&lt;&gt;"OK"),"Solo cable Ethernet",IF(AND($G23="KO",$H23="KO"),"Sin acceso","Pendiente"))))))</f>
-        <v>Sin acceso</v>
-      </c>
-      <c r="J23" s="59" t="s">
-        <v>83</v>
-      </c>
-      <c r="K23" s="61"/>
-      <c r="L23" s="62"/>
-      <c r="M23" s="59" t="s">
-        <v>38</v>
-      </c>
-      <c r="N23" s="63" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="48" t="str">
-        <f aca="false">IF($B24="","",ROW()-6)</f>
-        <v/>
-      </c>
-      <c r="B24" s="50"/>
-      <c r="C24" s="50"/>
-      <c r="D24" s="50"/>
-      <c r="E24" s="50"/>
-      <c r="F24" s="43"/>
-      <c r="G24" s="43"/>
-      <c r="H24" s="43"/>
-      <c r="I24" s="52" t="str">
-        <f aca="false">IF($B24="","",IF($F24="No aplica","No aplica",IF(AND($G24="OK",$H24="OK"),"Acceso total (WiFi + Cable)",IF(AND($G24="OK",$H24&lt;&gt;"OK"),"Solo WiFi",IF(AND($H24="OK",$G24&lt;&gt;"OK"),"Solo cable Ethernet",IF(AND($G24="KO",$H24="KO"),"Sin acceso","Pendiente"))))))</f>
-        <v/>
-      </c>
-      <c r="J24" s="43"/>
-      <c r="K24" s="45"/>
-      <c r="L24" s="46"/>
-      <c r="M24" s="43"/>
-      <c r="N24" s="47"/>
-    </row>
-    <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="K24" s="63"/>
+      <c r="L24" s="64"/>
+      <c r="M24" s="60" t="s">
+        <v>34</v>
+      </c>
+      <c r="N24" s="65"/>
+    </row>
+    <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="39" t="str">
         <f aca="false">IF($B25="","",ROW()-6)</f>
         <v/>
@@ -4772,20 +4828,20 @@
       <c r="C25" s="41"/>
       <c r="D25" s="41"/>
       <c r="E25" s="41"/>
-      <c r="F25" s="43"/>
+      <c r="F25" s="42"/>
       <c r="G25" s="43"/>
       <c r="H25" s="43"/>
       <c r="I25" s="44" t="str">
-        <f aca="false">IF($B25="","",IF($F25="No aplica","No aplica",IF(AND($G25="OK",$H25="OK"),"Acceso total (WiFi + Cable)",IF(AND($G25="OK",$H25&lt;&gt;"OK"),"Solo WiFi",IF(AND($H25="OK",$G25&lt;&gt;"OK"),"Solo cable Ethernet",IF(AND($G25="KO",$H25="KO"),"Sin acceso","Pendiente"))))))</f>
+        <f aca="false">IF($B25="","",IF($F25="No aplica","No aplica",IF(AND($G25="OK",$H25="OK"),"WiFi y cable",IF(AND($G25="OK",$H25&lt;&gt;"OK"),"Solo WiFi",IF(AND($H25="OK",$G25&lt;&gt;"OK"),"Solo cable",IF(AND($G25="KO",$H25="KO"),"Sin acceso","Pendiente"))))))</f>
         <v/>
       </c>
       <c r="J25" s="43"/>
       <c r="K25" s="45"/>
       <c r="L25" s="46"/>
-      <c r="M25" s="43"/>
+      <c r="M25" s="42"/>
       <c r="N25" s="47"/>
     </row>
-    <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="48" t="str">
         <f aca="false">IF($B26="","",ROW()-6)</f>
         <v/>
@@ -4794,20 +4850,20 @@
       <c r="C26" s="50"/>
       <c r="D26" s="50"/>
       <c r="E26" s="50"/>
-      <c r="F26" s="43"/>
+      <c r="F26" s="42"/>
       <c r="G26" s="43"/>
       <c r="H26" s="43"/>
       <c r="I26" s="52" t="str">
-        <f aca="false">IF($B26="","",IF($F26="No aplica","No aplica",IF(AND($G26="OK",$H26="OK"),"Acceso total (WiFi + Cable)",IF(AND($G26="OK",$H26&lt;&gt;"OK"),"Solo WiFi",IF(AND($H26="OK",$G26&lt;&gt;"OK"),"Solo cable Ethernet",IF(AND($G26="KO",$H26="KO"),"Sin acceso","Pendiente"))))))</f>
+        <f aca="false">IF($B26="","",IF($F26="No aplica","No aplica",IF(AND($G26="OK",$H26="OK"),"WiFi y cable",IF(AND($G26="OK",$H26&lt;&gt;"OK"),"Solo WiFi",IF(AND($H26="OK",$G26&lt;&gt;"OK"),"Solo cable",IF(AND($G26="KO",$H26="KO"),"Sin acceso","Pendiente"))))))</f>
         <v/>
       </c>
       <c r="J26" s="43"/>
       <c r="K26" s="45"/>
       <c r="L26" s="46"/>
-      <c r="M26" s="43"/>
+      <c r="M26" s="42"/>
       <c r="N26" s="47"/>
     </row>
-    <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="39" t="str">
         <f aca="false">IF($B27="","",ROW()-6)</f>
         <v/>
@@ -4816,20 +4872,20 @@
       <c r="C27" s="41"/>
       <c r="D27" s="41"/>
       <c r="E27" s="41"/>
-      <c r="F27" s="43"/>
+      <c r="F27" s="42"/>
       <c r="G27" s="43"/>
       <c r="H27" s="43"/>
       <c r="I27" s="44" t="str">
-        <f aca="false">IF($B27="","",IF($F27="No aplica","No aplica",IF(AND($G27="OK",$H27="OK"),"Acceso total (WiFi + Cable)",IF(AND($G27="OK",$H27&lt;&gt;"OK"),"Solo WiFi",IF(AND($H27="OK",$G27&lt;&gt;"OK"),"Solo cable Ethernet",IF(AND($G27="KO",$H27="KO"),"Sin acceso","Pendiente"))))))</f>
+        <f aca="false">IF($B27="","",IF($F27="No aplica","No aplica",IF(AND($G27="OK",$H27="OK"),"WiFi y cable",IF(AND($G27="OK",$H27&lt;&gt;"OK"),"Solo WiFi",IF(AND($H27="OK",$G27&lt;&gt;"OK"),"Solo cable",IF(AND($G27="KO",$H27="KO"),"Sin acceso","Pendiente"))))))</f>
         <v/>
       </c>
       <c r="J27" s="43"/>
       <c r="K27" s="45"/>
       <c r="L27" s="46"/>
-      <c r="M27" s="43"/>
+      <c r="M27" s="42"/>
       <c r="N27" s="47"/>
     </row>
-    <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="48" t="str">
         <f aca="false">IF($B28="","",ROW()-6)</f>
         <v/>
@@ -4838,20 +4894,20 @@
       <c r="C28" s="50"/>
       <c r="D28" s="50"/>
       <c r="E28" s="50"/>
-      <c r="F28" s="43"/>
+      <c r="F28" s="42"/>
       <c r="G28" s="43"/>
       <c r="H28" s="43"/>
       <c r="I28" s="52" t="str">
-        <f aca="false">IF($B28="","",IF($F28="No aplica","No aplica",IF(AND($G28="OK",$H28="OK"),"Acceso total (WiFi + Cable)",IF(AND($G28="OK",$H28&lt;&gt;"OK"),"Solo WiFi",IF(AND($H28="OK",$G28&lt;&gt;"OK"),"Solo cable Ethernet",IF(AND($G28="KO",$H28="KO"),"Sin acceso","Pendiente"))))))</f>
+        <f aca="false">IF($B28="","",IF($F28="No aplica","No aplica",IF(AND($G28="OK",$H28="OK"),"WiFi y cable",IF(AND($G28="OK",$H28&lt;&gt;"OK"),"Solo WiFi",IF(AND($H28="OK",$G28&lt;&gt;"OK"),"Solo cable",IF(AND($G28="KO",$H28="KO"),"Sin acceso","Pendiente"))))))</f>
         <v/>
       </c>
       <c r="J28" s="43"/>
       <c r="K28" s="45"/>
       <c r="L28" s="46"/>
-      <c r="M28" s="43"/>
+      <c r="M28" s="42"/>
       <c r="N28" s="47"/>
     </row>
-    <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="39" t="str">
         <f aca="false">IF($B29="","",ROW()-6)</f>
         <v/>
@@ -4860,20 +4916,20 @@
       <c r="C29" s="41"/>
       <c r="D29" s="41"/>
       <c r="E29" s="41"/>
-      <c r="F29" s="43"/>
+      <c r="F29" s="42"/>
       <c r="G29" s="43"/>
       <c r="H29" s="43"/>
       <c r="I29" s="44" t="str">
-        <f aca="false">IF($B29="","",IF($F29="No aplica","No aplica",IF(AND($G29="OK",$H29="OK"),"Acceso total (WiFi + Cable)",IF(AND($G29="OK",$H29&lt;&gt;"OK"),"Solo WiFi",IF(AND($H29="OK",$G29&lt;&gt;"OK"),"Solo cable Ethernet",IF(AND($G29="KO",$H29="KO"),"Sin acceso","Pendiente"))))))</f>
+        <f aca="false">IF($B29="","",IF($F29="No aplica","No aplica",IF(AND($G29="OK",$H29="OK"),"WiFi y cable",IF(AND($G29="OK",$H29&lt;&gt;"OK"),"Solo WiFi",IF(AND($H29="OK",$G29&lt;&gt;"OK"),"Solo cable",IF(AND($G29="KO",$H29="KO"),"Sin acceso","Pendiente"))))))</f>
         <v/>
       </c>
       <c r="J29" s="43"/>
       <c r="K29" s="45"/>
       <c r="L29" s="46"/>
-      <c r="M29" s="43"/>
+      <c r="M29" s="42"/>
       <c r="N29" s="47"/>
     </row>
-    <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="48" t="str">
         <f aca="false">IF($B30="","",ROW()-6)</f>
         <v/>
@@ -4882,20 +4938,20 @@
       <c r="C30" s="50"/>
       <c r="D30" s="50"/>
       <c r="E30" s="50"/>
-      <c r="F30" s="43"/>
+      <c r="F30" s="42"/>
       <c r="G30" s="43"/>
       <c r="H30" s="43"/>
       <c r="I30" s="52" t="str">
-        <f aca="false">IF($B30="","",IF($F30="No aplica","No aplica",IF(AND($G30="OK",$H30="OK"),"Acceso total (WiFi + Cable)",IF(AND($G30="OK",$H30&lt;&gt;"OK"),"Solo WiFi",IF(AND($H30="OK",$G30&lt;&gt;"OK"),"Solo cable Ethernet",IF(AND($G30="KO",$H30="KO"),"Sin acceso","Pendiente"))))))</f>
+        <f aca="false">IF($B30="","",IF($F30="No aplica","No aplica",IF(AND($G30="OK",$H30="OK"),"WiFi y cable",IF(AND($G30="OK",$H30&lt;&gt;"OK"),"Solo WiFi",IF(AND($H30="OK",$G30&lt;&gt;"OK"),"Solo cable",IF(AND($G30="KO",$H30="KO"),"Sin acceso","Pendiente"))))))</f>
         <v/>
       </c>
       <c r="J30" s="43"/>
       <c r="K30" s="45"/>
       <c r="L30" s="46"/>
-      <c r="M30" s="43"/>
+      <c r="M30" s="42"/>
       <c r="N30" s="47"/>
     </row>
-    <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="39" t="str">
         <f aca="false">IF($B31="","",ROW()-6)</f>
         <v/>
@@ -4904,20 +4960,20 @@
       <c r="C31" s="41"/>
       <c r="D31" s="41"/>
       <c r="E31" s="41"/>
-      <c r="F31" s="43"/>
+      <c r="F31" s="42"/>
       <c r="G31" s="43"/>
       <c r="H31" s="43"/>
       <c r="I31" s="44" t="str">
-        <f aca="false">IF($B31="","",IF($F31="No aplica","No aplica",IF(AND($G31="OK",$H31="OK"),"Acceso total (WiFi + Cable)",IF(AND($G31="OK",$H31&lt;&gt;"OK"),"Solo WiFi",IF(AND($H31="OK",$G31&lt;&gt;"OK"),"Solo cable Ethernet",IF(AND($G31="KO",$H31="KO"),"Sin acceso","Pendiente"))))))</f>
+        <f aca="false">IF($B31="","",IF($F31="No aplica","No aplica",IF(AND($G31="OK",$H31="OK"),"WiFi y cable",IF(AND($G31="OK",$H31&lt;&gt;"OK"),"Solo WiFi",IF(AND($H31="OK",$G31&lt;&gt;"OK"),"Solo cable",IF(AND($G31="KO",$H31="KO"),"Sin acceso","Pendiente"))))))</f>
         <v/>
       </c>
       <c r="J31" s="43"/>
       <c r="K31" s="45"/>
       <c r="L31" s="46"/>
-      <c r="M31" s="43"/>
+      <c r="M31" s="42"/>
       <c r="N31" s="47"/>
     </row>
-    <row r="32" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="48" t="str">
         <f aca="false">IF($B32="","",ROW()-6)</f>
         <v/>
@@ -4926,231 +4982,253 @@
       <c r="C32" s="50"/>
       <c r="D32" s="50"/>
       <c r="E32" s="50"/>
-      <c r="F32" s="43"/>
+      <c r="F32" s="42"/>
       <c r="G32" s="43"/>
       <c r="H32" s="43"/>
       <c r="I32" s="52" t="str">
-        <f aca="false">IF($B32="","",IF($F32="No aplica","No aplica",IF(AND($G32="OK",$H32="OK"),"Acceso total (WiFi + Cable)",IF(AND($G32="OK",$H32&lt;&gt;"OK"),"Solo WiFi",IF(AND($H32="OK",$G32&lt;&gt;"OK"),"Solo cable Ethernet",IF(AND($G32="KO",$H32="KO"),"Sin acceso","Pendiente"))))))</f>
+        <f aca="false">IF($B32="","",IF($F32="No aplica","No aplica",IF(AND($G32="OK",$H32="OK"),"WiFi y cable",IF(AND($G32="OK",$H32&lt;&gt;"OK"),"Solo WiFi",IF(AND($H32="OK",$G32&lt;&gt;"OK"),"Solo cable",IF(AND($G32="KO",$H32="KO"),"Sin acceso","Pendiente"))))))</f>
         <v/>
       </c>
       <c r="J32" s="43"/>
       <c r="K32" s="45"/>
       <c r="L32" s="46"/>
-      <c r="M32" s="43"/>
+      <c r="M32" s="42"/>
       <c r="N32" s="47"/>
     </row>
-    <row r="33" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="64" t="str">
+    <row r="33" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="39" t="str">
         <f aca="false">IF($B33="","",ROW()-6)</f>
         <v/>
       </c>
-      <c r="B33" s="65"/>
-      <c r="C33" s="65"/>
-      <c r="D33" s="65"/>
-      <c r="E33" s="65"/>
-      <c r="F33" s="66"/>
-      <c r="G33" s="66"/>
-      <c r="H33" s="66"/>
-      <c r="I33" s="67" t="str">
-        <f aca="false">IF($B33="","",IF($F33="No aplica","No aplica",IF(AND($G33="OK",$H33="OK"),"Acceso total (WiFi + Cable)",IF(AND($G33="OK",$H33&lt;&gt;"OK"),"Solo WiFi",IF(AND($H33="OK",$G33&lt;&gt;"OK"),"Solo cable Ethernet",IF(AND($G33="KO",$H33="KO"),"Sin acceso","Pendiente"))))))</f>
+      <c r="B33" s="41"/>
+      <c r="C33" s="41"/>
+      <c r="D33" s="41"/>
+      <c r="E33" s="41"/>
+      <c r="F33" s="42"/>
+      <c r="G33" s="43"/>
+      <c r="H33" s="43"/>
+      <c r="I33" s="44" t="str">
+        <f aca="false">IF($B33="","",IF($F33="No aplica","No aplica",IF(AND($G33="OK",$H33="OK"),"WiFi y cable",IF(AND($G33="OK",$H33&lt;&gt;"OK"),"Solo WiFi",IF(AND($H33="OK",$G33&lt;&gt;"OK"),"Solo cable",IF(AND($G33="KO",$H33="KO"),"Sin acceso","Pendiente"))))))</f>
         <v/>
       </c>
-      <c r="J33" s="66"/>
-      <c r="K33" s="68"/>
-      <c r="L33" s="69"/>
-      <c r="M33" s="66"/>
-      <c r="N33" s="70"/>
-    </row>
-    <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="71" t="s">
+      <c r="J33" s="43"/>
+      <c r="K33" s="45"/>
+      <c r="L33" s="46"/>
+      <c r="M33" s="42"/>
+      <c r="N33" s="47"/>
+    </row>
+    <row r="34" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="66" t="str">
+        <f aca="false">IF($B34="","",ROW()-6)</f>
+        <v/>
+      </c>
+      <c r="B34" s="67"/>
+      <c r="C34" s="67"/>
+      <c r="D34" s="67"/>
+      <c r="E34" s="67"/>
+      <c r="F34" s="68"/>
+      <c r="G34" s="69"/>
+      <c r="H34" s="69"/>
+      <c r="I34" s="70" t="str">
+        <f aca="false">IF($B34="","",IF($F34="No aplica","No aplica",IF(AND($G34="OK",$H34="OK"),"WiFi y cable",IF(AND($G34="OK",$H34&lt;&gt;"OK"),"Solo WiFi",IF(AND($H34="OK",$G34&lt;&gt;"OK"),"Solo cable",IF(AND($G34="KO",$H34="KO"),"Sin acceso","Pendiente"))))))</f>
+        <v/>
+      </c>
+      <c r="J34" s="69"/>
+      <c r="K34" s="71"/>
+      <c r="L34" s="72"/>
+      <c r="M34" s="68"/>
+      <c r="N34" s="73"/>
+    </row>
+    <row r="36" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="74" t="s">
+        <v>119</v>
+      </c>
+      <c r="B36" s="74"/>
+      <c r="C36" s="74"/>
+      <c r="D36" s="74"/>
+      <c r="E36" s="74"/>
+      <c r="F36" s="74"/>
+      <c r="G36" s="74"/>
+      <c r="H36" s="74"/>
+      <c r="I36" s="74"/>
+      <c r="J36" s="74"/>
+      <c r="K36" s="74"/>
+      <c r="L36" s="74"/>
+      <c r="M36" s="74"/>
+      <c r="N36" s="74"/>
+    </row>
+    <row r="37" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="75" t="s">
+        <v>120</v>
+      </c>
+      <c r="B37" s="76" t="s">
+        <v>121</v>
+      </c>
+      <c r="C37" s="76" t="s">
+        <v>24</v>
+      </c>
+      <c r="D37" s="76" t="s">
+        <v>90</v>
+      </c>
+      <c r="E37" s="76" t="s">
+        <v>122</v>
+      </c>
+      <c r="F37" s="77" t="s">
+        <v>63</v>
+      </c>
+      <c r="G37" s="75" t="s">
+        <v>64</v>
+      </c>
+      <c r="H37" s="75" t="s">
+        <v>76</v>
+      </c>
+      <c r="I37" s="78" t="s">
+        <v>13</v>
+      </c>
+      <c r="J37" s="75" t="s">
+        <v>81</v>
+      </c>
+      <c r="K37" s="79" t="s">
+        <v>123</v>
+      </c>
+      <c r="L37" s="75" t="s">
+        <v>124</v>
+      </c>
+      <c r="M37" s="77" t="s">
+        <v>35</v>
+      </c>
+      <c r="N37" s="76" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="80" t="s">
         <v>126</v>
       </c>
-      <c r="B35" s="71"/>
-      <c r="C35" s="71"/>
-      <c r="D35" s="71"/>
-      <c r="E35" s="71"/>
-      <c r="F35" s="71"/>
-      <c r="G35" s="71"/>
-      <c r="H35" s="71"/>
-      <c r="I35" s="71"/>
-      <c r="J35" s="71"/>
-      <c r="K35" s="71"/>
-      <c r="L35" s="71"/>
-      <c r="M35" s="71"/>
-      <c r="N35" s="71"/>
-    </row>
-    <row r="36" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="72" t="s">
+      <c r="B39" s="80"/>
+      <c r="C39" s="80"/>
+      <c r="D39" s="80"/>
+      <c r="E39" s="80"/>
+      <c r="F39" s="80"/>
+      <c r="G39" s="80"/>
+      <c r="H39" s="80"/>
+      <c r="I39" s="80"/>
+      <c r="J39" s="80"/>
+      <c r="K39" s="80"/>
+      <c r="L39" s="80"/>
+      <c r="M39" s="80"/>
+      <c r="N39" s="80"/>
+    </row>
+    <row r="40" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="81" t="s">
         <v>127</v>
       </c>
-      <c r="B36" s="73" t="s">
+      <c r="B40" s="81"/>
+      <c r="C40" s="81"/>
+      <c r="D40" s="81"/>
+      <c r="E40" s="81"/>
+      <c r="F40" s="81"/>
+      <c r="G40" s="81"/>
+      <c r="H40" s="81"/>
+      <c r="I40" s="81"/>
+      <c r="J40" s="81"/>
+      <c r="K40" s="81"/>
+      <c r="L40" s="81"/>
+      <c r="M40" s="81"/>
+      <c r="N40" s="81"/>
+    </row>
+    <row r="41" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="81" t="s">
         <v>128</v>
       </c>
-      <c r="C36" s="73" t="s">
-        <v>22</v>
-      </c>
-      <c r="D36" s="73" t="s">
-        <v>93</v>
-      </c>
-      <c r="E36" s="73" t="s">
+      <c r="B41" s="81"/>
+      <c r="C41" s="81"/>
+      <c r="D41" s="81"/>
+      <c r="E41" s="81"/>
+      <c r="F41" s="81"/>
+      <c r="G41" s="81"/>
+      <c r="H41" s="81"/>
+      <c r="I41" s="81"/>
+      <c r="J41" s="81"/>
+      <c r="K41" s="81"/>
+      <c r="L41" s="81"/>
+      <c r="M41" s="81"/>
+      <c r="N41" s="81"/>
+    </row>
+    <row r="42" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="81" t="s">
         <v>129</v>
       </c>
-      <c r="F36" s="72" t="s">
-        <v>76</v>
-      </c>
-      <c r="G36" s="72" t="s">
-        <v>77</v>
-      </c>
-      <c r="H36" s="72" t="s">
-        <v>78</v>
-      </c>
-      <c r="I36" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="J36" s="72" t="s">
-        <v>83</v>
-      </c>
-      <c r="K36" s="75" t="s">
+      <c r="B42" s="81"/>
+      <c r="C42" s="81"/>
+      <c r="D42" s="81"/>
+      <c r="E42" s="81"/>
+      <c r="F42" s="81"/>
+      <c r="G42" s="81"/>
+      <c r="H42" s="81"/>
+      <c r="I42" s="81"/>
+      <c r="J42" s="81"/>
+      <c r="K42" s="81"/>
+      <c r="L42" s="81"/>
+      <c r="M42" s="81"/>
+      <c r="N42" s="81"/>
+    </row>
+    <row r="43" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="81" t="s">
         <v>130</v>
       </c>
-      <c r="L36" s="72" t="s">
+      <c r="B43" s="81"/>
+      <c r="C43" s="81"/>
+      <c r="D43" s="81"/>
+      <c r="E43" s="81"/>
+      <c r="F43" s="81"/>
+      <c r="G43" s="81"/>
+      <c r="H43" s="81"/>
+      <c r="I43" s="81"/>
+      <c r="J43" s="81"/>
+      <c r="K43" s="81"/>
+      <c r="L43" s="81"/>
+      <c r="M43" s="81"/>
+      <c r="N43" s="81"/>
+    </row>
+    <row r="44" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="81" t="s">
         <v>131</v>
       </c>
-      <c r="M36" s="72" t="s">
-        <v>39</v>
-      </c>
-      <c r="N36" s="73" t="s">
+      <c r="B44" s="81"/>
+      <c r="C44" s="81"/>
+      <c r="D44" s="81"/>
+      <c r="E44" s="81"/>
+      <c r="F44" s="81"/>
+      <c r="G44" s="81"/>
+      <c r="H44" s="81"/>
+      <c r="I44" s="81"/>
+      <c r="J44" s="81"/>
+      <c r="K44" s="81"/>
+      <c r="L44" s="81"/>
+      <c r="M44" s="81"/>
+      <c r="N44" s="81"/>
+    </row>
+    <row r="45" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="81" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="38" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="76" t="s">
-        <v>133</v>
-      </c>
-      <c r="B38" s="76"/>
-      <c r="C38" s="76"/>
-      <c r="D38" s="76"/>
-      <c r="E38" s="76"/>
-      <c r="F38" s="76"/>
-      <c r="G38" s="76"/>
-      <c r="H38" s="76"/>
-      <c r="I38" s="76"/>
-      <c r="J38" s="76"/>
-      <c r="K38" s="76"/>
-      <c r="L38" s="76"/>
-      <c r="M38" s="76"/>
-      <c r="N38" s="76"/>
-    </row>
-    <row r="39" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="77" t="s">
-        <v>134</v>
-      </c>
-      <c r="B39" s="77"/>
-      <c r="C39" s="77"/>
-      <c r="D39" s="77"/>
-      <c r="E39" s="77"/>
-      <c r="F39" s="77"/>
-      <c r="G39" s="77"/>
-      <c r="H39" s="77"/>
-      <c r="I39" s="77"/>
-      <c r="J39" s="77"/>
-      <c r="K39" s="77"/>
-      <c r="L39" s="77"/>
-      <c r="M39" s="77"/>
-      <c r="N39" s="77"/>
-    </row>
-    <row r="40" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="77" t="s">
-        <v>135</v>
-      </c>
-      <c r="B40" s="77"/>
-      <c r="C40" s="77"/>
-      <c r="D40" s="77"/>
-      <c r="E40" s="77"/>
-      <c r="F40" s="77"/>
-      <c r="G40" s="77"/>
-      <c r="H40" s="77"/>
-      <c r="I40" s="77"/>
-      <c r="J40" s="77"/>
-      <c r="K40" s="77"/>
-      <c r="L40" s="77"/>
-      <c r="M40" s="77"/>
-      <c r="N40" s="77"/>
-    </row>
-    <row r="41" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="77" t="s">
-        <v>136</v>
-      </c>
-      <c r="B41" s="77"/>
-      <c r="C41" s="77"/>
-      <c r="D41" s="77"/>
-      <c r="E41" s="77"/>
-      <c r="F41" s="77"/>
-      <c r="G41" s="77"/>
-      <c r="H41" s="77"/>
-      <c r="I41" s="77"/>
-      <c r="J41" s="77"/>
-      <c r="K41" s="77"/>
-      <c r="L41" s="77"/>
-      <c r="M41" s="77"/>
-      <c r="N41" s="77"/>
-    </row>
-    <row r="42" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="77" t="s">
-        <v>137</v>
-      </c>
-      <c r="B42" s="77"/>
-      <c r="C42" s="77"/>
-      <c r="D42" s="77"/>
-      <c r="E42" s="77"/>
-      <c r="F42" s="77"/>
-      <c r="G42" s="77"/>
-      <c r="H42" s="77"/>
-      <c r="I42" s="77"/>
-      <c r="J42" s="77"/>
-      <c r="K42" s="77"/>
-      <c r="L42" s="77"/>
-      <c r="M42" s="77"/>
-      <c r="N42" s="77"/>
-    </row>
-    <row r="43" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="77" t="s">
-        <v>138</v>
-      </c>
-      <c r="B43" s="77"/>
-      <c r="C43" s="77"/>
-      <c r="D43" s="77"/>
-      <c r="E43" s="77"/>
-      <c r="F43" s="77"/>
-      <c r="G43" s="77"/>
-      <c r="H43" s="77"/>
-      <c r="I43" s="77"/>
-      <c r="J43" s="77"/>
-      <c r="K43" s="77"/>
-      <c r="L43" s="77"/>
-      <c r="M43" s="77"/>
-      <c r="N43" s="77"/>
-    </row>
-    <row r="44" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="77" t="s">
-        <v>139</v>
-      </c>
-      <c r="B44" s="77"/>
-      <c r="C44" s="77"/>
-      <c r="D44" s="77"/>
-      <c r="E44" s="77"/>
-      <c r="F44" s="77"/>
-      <c r="G44" s="77"/>
-      <c r="H44" s="77"/>
-      <c r="I44" s="77"/>
-      <c r="J44" s="77"/>
-      <c r="K44" s="77"/>
-      <c r="L44" s="77"/>
-      <c r="M44" s="77"/>
-      <c r="N44" s="77"/>
+      <c r="B45" s="81"/>
+      <c r="C45" s="81"/>
+      <c r="D45" s="81"/>
+      <c r="E45" s="81"/>
+      <c r="F45" s="81"/>
+      <c r="G45" s="81"/>
+      <c r="H45" s="81"/>
+      <c r="I45" s="81"/>
+      <c r="J45" s="81"/>
+      <c r="K45" s="81"/>
+      <c r="L45" s="81"/>
+      <c r="M45" s="81"/>
+      <c r="N45" s="81"/>
     </row>
   </sheetData>
-  <autoFilter ref="A6:N33"/>
+  <autoFilter ref="A6:N34"/>
   <mergeCells count="17">
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="A2:N2"/>
@@ -5161,16 +5239,16 @@
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="I4:J4"/>
     <mergeCell ref="K4:N4"/>
-    <mergeCell ref="A35:N35"/>
-    <mergeCell ref="A38:N38"/>
+    <mergeCell ref="A36:N36"/>
     <mergeCell ref="A39:N39"/>
     <mergeCell ref="A40:N40"/>
     <mergeCell ref="A41:N41"/>
     <mergeCell ref="A42:N42"/>
     <mergeCell ref="A43:N43"/>
     <mergeCell ref="A44:N44"/>
+    <mergeCell ref="A45:N45"/>
   </mergeCells>
-  <conditionalFormatting sqref="G7:H33">
+  <conditionalFormatting sqref="G7:H34">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
       <formula>"OK"</formula>
     </cfRule>
@@ -5184,7 +5262,7 @@
       <formula>"N/A"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F7:F33">
+  <conditionalFormatting sqref="F7:F34">
     <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
       <formula>"Probado"</formula>
     </cfRule>
@@ -5201,15 +5279,15 @@
       <formula>"No aplica"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I7:I33">
+  <conditionalFormatting sqref="I7:I34">
     <cfRule type="cellIs" priority="11" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
-      <formula>"Acceso total (WiFi + Cable)"</formula>
+      <formula>"WiFi y cable"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="12" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="21">
       <formula>"Solo WiFi"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="13" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="21">
-      <formula>"Solo cable Ethernet"</formula>
+      <formula>"Solo cable"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="14" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
       <formula>"Sin acceso"</formula>
@@ -5221,7 +5299,7 @@
       <formula>"No aplica"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J7:J33">
+  <conditionalFormatting sqref="J7:J34">
     <cfRule type="cellIs" priority="17" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
       <formula>"Crítica"</formula>
     </cfRule>
@@ -5235,51 +5313,51 @@
       <formula>"Baja"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M7:M33">
+  <conditionalFormatting sqref="M7:M34">
     <cfRule type="cellIs" priority="21" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
       <formula>"Ninguna"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B7:B33">
+  <conditionalFormatting sqref="B7:B34">
     <cfRule type="expression" priority="22" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="23">
-      <formula>AND($J7="Crítica",$I7&lt;&gt;"Acceso total (WiFi + Cable)",$B7&lt;&gt;"")</formula>
+      <formula>AND($J7="Crítica",$I7&lt;&gt;"WiFi y cable",$B7&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="5">
-    <dataValidation allowBlank="true" error="Elija uno de los valores del desplegable (o amplíe la lista en la hoja «Listas»)." errorStyle="stop" errorTitle="Valor no válido" operator="between" prompt="Seleccione un valor de la lista desplegable." promptTitle="Estado de la prueba" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="F7:F33" type="list">
+    <dataValidation allowBlank="true" error="Usa uno de los valores de la lista, o amplíala en la hoja Listas." errorStyle="stop" errorTitle="Valor no válido" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F7:F34" type="list">
       <formula1>lst_Estado</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Elija uno de los valores del desplegable (o amplíe la lista en la hoja «Listas»)." errorStyle="stop" errorTitle="Valor no válido" operator="between" prompt="OK = con acceso · KO = sin acceso · No probado · N/A = no aplica." promptTitle="Resultado de la conexión" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="G7:H33" type="list">
+    <dataValidation allowBlank="true" error="Usa uno de los valores de la lista, o amplíala en la hoja Listas." errorStyle="stop" errorTitle="Valor no válido" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G7:H34" type="list">
       <formula1>lst_Conexion</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Elija uno de los valores del desplegable (o amplíe la lista en la hoja «Listas»)." errorStyle="stop" errorTitle="Valor no válido" operator="between" prompt="Impacto en el negocio si el sistema no está disponible." promptTitle="Criticidad" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="J7:J33" type="list">
+    <dataValidation allowBlank="true" error="Usa uno de los valores de la lista, o amplíala en la hoja Listas." errorStyle="stop" errorTitle="Valor no válido" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="J7:J34" type="list">
       <formula1>lst_Criticidad</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Elija uno de los valores del desplegable (o amplíe la lista en la hoja «Listas»)." errorStyle="stop" errorTitle="Valor no válido" operator="between" prompt="Siguiente paso para desbloquear o completar la prueba." promptTitle="Próxima acción" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="M7:M33" type="list">
+    <dataValidation allowBlank="true" error="Usa uno de los valores de la lista, o amplíala en la hoja Listas." errorStyle="stop" errorTitle="Valor no válido" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="M7:M34" type="list">
       <formula1>lst_Accion</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Introduzca una fecha válida (DD/MM/AAAA)." errorStyle="stop" errorTitle="Fecha no válida" operator="greaterThan" prompt="Formato DD/MM/AAAA." promptTitle="Fecha de prueba" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="L7:L33" type="date">
+    <dataValidation allowBlank="true" error="Formato DD/MM/AAAA." errorStyle="stop" errorTitle="Fecha no válida" operator="greaterThan" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="L7:L34" type="date">
       <formula1>DATE(2000,1,1)</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="E8" r:id="rId2" display="https://ipstorefront.ipaper.com/"/>
-    <hyperlink ref="E9" r:id="rId3" display="http://ub99sagep03:8124/auth/login/page"/>
-    <hyperlink ref="E10" r:id="rId4" display="https://ipapercloud.sharepoint.com/"/>
-    <hyperlink ref="E11" r:id="rId5" display="https://apps.powerapps.com/"/>
-    <hyperlink ref="E12" r:id="rId6" display="https://miacceso.e-factura.net/"/>
-    <hyperlink ref="E15" r:id="rId7" display="https://myaccess.ipaper.com/"/>
-    <hyperlink ref="E16" r:id="rId8" display="https://ocr.emea.ipaper.com/"/>
-    <hyperlink ref="E17" r:id="rId9" display="https://ecm.emea.ipaper.com/"/>
-    <hyperlink ref="E18" r:id="rId10" display="https://ap.xelix.com/login"/>
-    <hyperlink ref="E20" r:id="rId11" display="https://apupload.ipaper.com/"/>
-    <hyperlink ref="E21" r:id="rId12" display="https://bi.ipaper.com/BOE/BI/logonNoSso.jsp"/>
-    <hyperlink ref="E22" r:id="rId13" display="http://s02afnbgp03.na.ipaper.com/P8LoadViewer/"/>
+    <hyperlink ref="E9" r:id="rId2" display="https://ipstorefront.ipaper.com/"/>
+    <hyperlink ref="E10" r:id="rId3" display="http://ub99sagep03:8124/auth/login/page"/>
+    <hyperlink ref="E11" r:id="rId4" display="https://ipapercloud.sharepoint.com/"/>
+    <hyperlink ref="E12" r:id="rId5" display="https://apps.powerapps.com/"/>
+    <hyperlink ref="E13" r:id="rId6" display="https://miacceso.e-factura.net/"/>
+    <hyperlink ref="E16" r:id="rId7" display="https://myaccess.ipaper.com/"/>
+    <hyperlink ref="E17" r:id="rId8" display="https://ocr.emea.ipaper.com/"/>
+    <hyperlink ref="E18" r:id="rId9" display="https://ecm.emea.ipaper.com/"/>
+    <hyperlink ref="E19" r:id="rId10" display="https://ap.xelix.com/login"/>
+    <hyperlink ref="E21" r:id="rId11" display="https://apupload.ipaper.com/"/>
+    <hyperlink ref="E22" r:id="rId12" display="https://bi.ipaper.com/BOE/BI/logonNoSso.jsp"/>
+    <hyperlink ref="E23" r:id="rId13" display="http://s02afnbgp03.na.ipaper.com/P8LoadViewer/"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -5304,141 +5382,141 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2.5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="20"/>
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="78" t="s">
-        <v>140</v>
-      </c>
-      <c r="C2" s="78"/>
-      <c r="D2" s="78"/>
-      <c r="E2" s="78"/>
-      <c r="F2" s="78"/>
+      <c r="B2" s="82" t="s">
+        <v>133</v>
+      </c>
+      <c r="C2" s="82"/>
+      <c r="D2" s="82"/>
+      <c r="E2" s="82"/>
+      <c r="F2" s="82"/>
     </row>
     <row r="3" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="27" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="C3" s="27"/>
       <c r="D3" s="27"/>
       <c r="E3" s="27"/>
       <c r="F3" s="27"/>
     </row>
-    <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="79" t="s">
-        <v>59</v>
-      </c>
-      <c r="C5" s="79" t="s">
+    <row r="5" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B5" s="83" t="s">
+        <v>55</v>
+      </c>
+      <c r="C5" s="83" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" s="83" t="s">
+        <v>135</v>
+      </c>
+      <c r="E5" s="83" t="s">
+        <v>58</v>
+      </c>
+      <c r="F5" s="83" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="84" t="s">
+        <v>70</v>
+      </c>
+      <c r="C6" s="84" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" s="84" t="s">
+        <v>64</v>
+      </c>
+      <c r="E6" s="84" t="s">
+        <v>65</v>
+      </c>
+      <c r="F6" s="84" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="85" t="s">
+        <v>95</v>
+      </c>
+      <c r="C7" s="85" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" s="85" t="s">
+        <v>76</v>
+      </c>
+      <c r="E7" s="85" t="s">
+        <v>81</v>
+      </c>
+      <c r="F7" s="85" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="84" t="s">
+        <v>136</v>
+      </c>
+      <c r="C8" s="84" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="79" t="s">
-        <v>142</v>
-      </c>
-      <c r="E5" s="79" t="s">
-        <v>62</v>
-      </c>
-      <c r="F5" s="79" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="80" t="s">
-        <v>69</v>
-      </c>
-      <c r="C6" s="80" t="s">
+      <c r="D8" s="84" t="s">
+        <v>71</v>
+      </c>
+      <c r="E8" s="84" t="s">
+        <v>86</v>
+      </c>
+      <c r="F8" s="84" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="85" t="s">
+        <v>63</v>
+      </c>
+      <c r="C9" s="85" t="s">
+        <v>34</v>
+      </c>
+      <c r="D9" s="85" t="s">
+        <v>137</v>
+      </c>
+      <c r="E9" s="85" t="s">
+        <v>138</v>
+      </c>
+      <c r="F9" s="85" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="84" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="84" t="s">
         <v>35</v>
       </c>
-      <c r="D6" s="80" t="s">
-        <v>77</v>
-      </c>
-      <c r="E6" s="80" t="s">
-        <v>71</v>
-      </c>
-      <c r="F6" s="80" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="81" t="s">
-        <v>98</v>
-      </c>
-      <c r="C7" s="81" t="s">
+      <c r="F10" s="84" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C11" s="85" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="81" t="s">
-        <v>78</v>
-      </c>
-      <c r="E7" s="81" t="s">
-        <v>83</v>
-      </c>
-      <c r="F7" s="81" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="80" t="s">
-        <v>144</v>
-      </c>
-      <c r="C8" s="80" t="s">
+      <c r="F11" s="85" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C12" s="84" t="s">
         <v>37</v>
       </c>
-      <c r="D8" s="80" t="s">
-        <v>70</v>
-      </c>
-      <c r="E8" s="80" t="s">
-        <v>88</v>
-      </c>
-      <c r="F8" s="80" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="81" t="s">
-        <v>76</v>
-      </c>
-      <c r="C9" s="81" t="s">
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C13" s="85" t="s">
         <v>38</v>
-      </c>
-      <c r="D9" s="81" t="s">
-        <v>145</v>
-      </c>
-      <c r="E9" s="81" t="s">
-        <v>146</v>
-      </c>
-      <c r="F9" s="81" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="80" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" s="80" t="s">
-        <v>39</v>
-      </c>
-      <c r="F10" s="80" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C11" s="81" t="s">
-        <v>40</v>
-      </c>
-      <c r="F11" s="81" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C12" s="80" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C13" s="81" t="s">
-        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -5453,5 +5531,6 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>